<commit_message>
fix(raw-data): correct districts & sub-districts against verified geography reference
sub_districts.json (7453 -> 7436 rows):
- remove 42 stale/duplicate codes (old codes left after district splits + 2 junk rows: สมก๋าย, โคกแหลม)
- add 25 missing tambons (new Bangkok subdistricts and subdivided children)
- re-align Bueng Kan (province 38): attach correct tambon names to their proper codes
- fix 6 wrong English names, 5 Thai names, 5 postal codes (e.g. เสม็ด 20130->20000, บางเสาธง 10540->10570)

districts.json (930 -> 928 rows):
- remove 2 invalid rows (7074, 9077 — local-municipality artifacts, not amphoes)
- fix 4 swapped Bueng Kan district names (3802/3804/3805/3807)

Regenerate api/latest and formats from corrected raw data.
</commit_message>
<xml_diff>
--- a/formats/xlsx/districts.xlsx
+++ b/formats/xlsx/districts.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G931"/>
+  <dimension ref="A1:G929"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5058,7 +5058,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Khoa Khitchakut</t>
+          <t>Khao Khitchakut</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -6798,7 +6798,7 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>Nong Bunnak</t>
+          <t>Nong Bun Mak</t>
         </is>
       </c>
       <c r="D220" t="n">
@@ -7668,7 +7668,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Din Daeng</t>
+          <t>Non Din Daeng</t>
         </is>
       </c>
       <c r="D250" t="n">
@@ -10592,12 +10592,12 @@
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>เซกา</t>
+          <t>พรเจริญ</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>Seka</t>
+          <t>Phon Charoen</t>
         </is>
       </c>
       <c r="D351" t="n">
@@ -10650,12 +10650,12 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>พรเจริญ</t>
+          <t>เซกา</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>Phon Charoen</t>
+          <t>Seka</t>
         </is>
       </c>
       <c r="D353" t="n">
@@ -10679,12 +10679,12 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>ศรีวิไล</t>
+          <t>ปากคาด</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>Si Wilai</t>
+          <t>Pak Khat</t>
         </is>
       </c>
       <c r="D354" t="n">
@@ -10737,12 +10737,12 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>ปากคาด</t>
+          <t>ศรีวิไล</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>Pak Khat</t>
+          <t>Si Wilai</t>
         </is>
       </c>
       <c r="D356" t="n">
@@ -12279,7 +12279,7 @@
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>rachak-sinlapakhom</t>
+          <t>Prachaksinlapakhom</t>
         </is>
       </c>
       <c r="D409" t="n">
@@ -13091,7 +13091,7 @@
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>Kantharawichai</t>
+          <t>Chiang Yuen</t>
         </is>
       </c>
       <c r="D437" t="n">
@@ -21492,20 +21492,20 @@
     </row>
     <row r="727">
       <c r="A727" t="n">
-        <v>7074</v>
+        <v>7101</v>
       </c>
       <c r="B727" t="inlineStr">
         <is>
-          <t>ท้องถิ่นเทศบาลตำบลบ้านฆ้อง</t>
+          <t>เมืองกาญจนบุรี</t>
         </is>
       </c>
       <c r="C727" t="inlineStr">
         <is>
-          <t>Tet Saban Ban Kong</t>
+          <t>Mueang Kanchanaburi</t>
         </is>
       </c>
       <c r="D727" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E727" t="inlineStr">
         <is>
@@ -21521,16 +21521,16 @@
     </row>
     <row r="728">
       <c r="A728" t="n">
-        <v>7101</v>
+        <v>7102</v>
       </c>
       <c r="B728" t="inlineStr">
         <is>
-          <t>เมืองกาญจนบุรี</t>
+          <t>ไทรโยค</t>
         </is>
       </c>
       <c r="C728" t="inlineStr">
         <is>
-          <t>Mueang Kanchanaburi</t>
+          <t>Sai Yok</t>
         </is>
       </c>
       <c r="D728" t="n">
@@ -21550,16 +21550,16 @@
     </row>
     <row r="729">
       <c r="A729" t="n">
-        <v>7102</v>
+        <v>7103</v>
       </c>
       <c r="B729" t="inlineStr">
         <is>
-          <t>ไทรโยค</t>
+          <t>บ่อพลอย</t>
         </is>
       </c>
       <c r="C729" t="inlineStr">
         <is>
-          <t>Sai Yok</t>
+          <t>Bo Phloi</t>
         </is>
       </c>
       <c r="D729" t="n">
@@ -21579,16 +21579,16 @@
     </row>
     <row r="730">
       <c r="A730" t="n">
-        <v>7103</v>
+        <v>7104</v>
       </c>
       <c r="B730" t="inlineStr">
         <is>
-          <t>บ่อพลอย</t>
+          <t>ศรีสวัสดิ์</t>
         </is>
       </c>
       <c r="C730" t="inlineStr">
         <is>
-          <t>Bo Phloi</t>
+          <t>Si Sawat</t>
         </is>
       </c>
       <c r="D730" t="n">
@@ -21608,16 +21608,16 @@
     </row>
     <row r="731">
       <c r="A731" t="n">
-        <v>7104</v>
+        <v>7105</v>
       </c>
       <c r="B731" t="inlineStr">
         <is>
-          <t>ศรีสวัสดิ์</t>
+          <t>ท่ามะกา</t>
         </is>
       </c>
       <c r="C731" t="inlineStr">
         <is>
-          <t>Si Sawat</t>
+          <t>Tha Maka</t>
         </is>
       </c>
       <c r="D731" t="n">
@@ -21637,16 +21637,16 @@
     </row>
     <row r="732">
       <c r="A732" t="n">
-        <v>7105</v>
+        <v>7106</v>
       </c>
       <c r="B732" t="inlineStr">
         <is>
-          <t>ท่ามะกา</t>
+          <t>ท่าม่วง</t>
         </is>
       </c>
       <c r="C732" t="inlineStr">
         <is>
-          <t>Tha Maka</t>
+          <t>Tha Muang</t>
         </is>
       </c>
       <c r="D732" t="n">
@@ -21666,16 +21666,16 @@
     </row>
     <row r="733">
       <c r="A733" t="n">
-        <v>7106</v>
+        <v>7107</v>
       </c>
       <c r="B733" t="inlineStr">
         <is>
-          <t>ท่าม่วง</t>
+          <t>ทองผาภูมิ</t>
         </is>
       </c>
       <c r="C733" t="inlineStr">
         <is>
-          <t>Tha Muang</t>
+          <t>Pha Phum</t>
         </is>
       </c>
       <c r="D733" t="n">
@@ -21695,16 +21695,16 @@
     </row>
     <row r="734">
       <c r="A734" t="n">
-        <v>7107</v>
+        <v>7108</v>
       </c>
       <c r="B734" t="inlineStr">
         <is>
-          <t>ทองผาภูมิ</t>
+          <t>สังขละบุรี</t>
         </is>
       </c>
       <c r="C734" t="inlineStr">
         <is>
-          <t>Pha Phum</t>
+          <t>Sangkhla Buri</t>
         </is>
       </c>
       <c r="D734" t="n">
@@ -21724,16 +21724,16 @@
     </row>
     <row r="735">
       <c r="A735" t="n">
-        <v>7108</v>
+        <v>7109</v>
       </c>
       <c r="B735" t="inlineStr">
         <is>
-          <t>สังขละบุรี</t>
+          <t>พนมทวน</t>
         </is>
       </c>
       <c r="C735" t="inlineStr">
         <is>
-          <t>Sangkhla Buri</t>
+          <t>Phanom Thuan</t>
         </is>
       </c>
       <c r="D735" t="n">
@@ -21753,16 +21753,16 @@
     </row>
     <row r="736">
       <c r="A736" t="n">
-        <v>7109</v>
+        <v>7110</v>
       </c>
       <c r="B736" t="inlineStr">
         <is>
-          <t>พนมทวน</t>
+          <t>เลาขวัญ</t>
         </is>
       </c>
       <c r="C736" t="inlineStr">
         <is>
-          <t>Phanom Thuan</t>
+          <t>Lao Khwan</t>
         </is>
       </c>
       <c r="D736" t="n">
@@ -21782,16 +21782,16 @@
     </row>
     <row r="737">
       <c r="A737" t="n">
-        <v>7110</v>
+        <v>7111</v>
       </c>
       <c r="B737" t="inlineStr">
         <is>
-          <t>เลาขวัญ</t>
+          <t>ด่านมะขามเตี้ย</t>
         </is>
       </c>
       <c r="C737" t="inlineStr">
         <is>
-          <t>Lao Khwan</t>
+          <t>Dan Makham Tia</t>
         </is>
       </c>
       <c r="D737" t="n">
@@ -21811,16 +21811,16 @@
     </row>
     <row r="738">
       <c r="A738" t="n">
-        <v>7111</v>
+        <v>7112</v>
       </c>
       <c r="B738" t="inlineStr">
         <is>
-          <t>ด่านมะขามเตี้ย</t>
+          <t>หนองปรือ</t>
         </is>
       </c>
       <c r="C738" t="inlineStr">
         <is>
-          <t>Dan Makham Tia</t>
+          <t>Nong Prue</t>
         </is>
       </c>
       <c r="D738" t="n">
@@ -21840,16 +21840,16 @@
     </row>
     <row r="739">
       <c r="A739" t="n">
-        <v>7112</v>
+        <v>7113</v>
       </c>
       <c r="B739" t="inlineStr">
         <is>
-          <t>หนองปรือ</t>
+          <t>ห้วยกระเจา</t>
         </is>
       </c>
       <c r="C739" t="inlineStr">
         <is>
-          <t>Nong Prue</t>
+          <t>Huai Krachao</t>
         </is>
       </c>
       <c r="D739" t="n">
@@ -21869,20 +21869,20 @@
     </row>
     <row r="740">
       <c r="A740" t="n">
-        <v>7113</v>
+        <v>7201</v>
       </c>
       <c r="B740" t="inlineStr">
         <is>
-          <t>ห้วยกระเจา</t>
+          <t>เมืองสุพรรณบุรี</t>
         </is>
       </c>
       <c r="C740" t="inlineStr">
         <is>
-          <t>Huai Krachao</t>
+          <t>Mueang Suphan Buri</t>
         </is>
       </c>
       <c r="D740" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E740" t="inlineStr">
         <is>
@@ -21898,16 +21898,16 @@
     </row>
     <row r="741">
       <c r="A741" t="n">
-        <v>7201</v>
+        <v>7202</v>
       </c>
       <c r="B741" t="inlineStr">
         <is>
-          <t>เมืองสุพรรณบุรี</t>
+          <t>เดิมบางนางบวช</t>
         </is>
       </c>
       <c r="C741" t="inlineStr">
         <is>
-          <t>Mueang Suphan Buri</t>
+          <t>Doem Bang Nang Buat</t>
         </is>
       </c>
       <c r="D741" t="n">
@@ -21927,16 +21927,16 @@
     </row>
     <row r="742">
       <c r="A742" t="n">
-        <v>7202</v>
+        <v>7203</v>
       </c>
       <c r="B742" t="inlineStr">
         <is>
-          <t>เดิมบางนางบวช</t>
+          <t>ด่านช้าง</t>
         </is>
       </c>
       <c r="C742" t="inlineStr">
         <is>
-          <t>Doem Bang Nang Buat</t>
+          <t>Dan Chang</t>
         </is>
       </c>
       <c r="D742" t="n">
@@ -21956,16 +21956,16 @@
     </row>
     <row r="743">
       <c r="A743" t="n">
-        <v>7203</v>
+        <v>7204</v>
       </c>
       <c r="B743" t="inlineStr">
         <is>
-          <t>ด่านช้าง</t>
+          <t>บางปลาม้า</t>
         </is>
       </c>
       <c r="C743" t="inlineStr">
         <is>
-          <t>Dan Chang</t>
+          <t>Bang Pla Ma</t>
         </is>
       </c>
       <c r="D743" t="n">
@@ -21985,16 +21985,16 @@
     </row>
     <row r="744">
       <c r="A744" t="n">
-        <v>7204</v>
+        <v>7205</v>
       </c>
       <c r="B744" t="inlineStr">
         <is>
-          <t>บางปลาม้า</t>
+          <t>ศรีประจันต์</t>
         </is>
       </c>
       <c r="C744" t="inlineStr">
         <is>
-          <t>Bang Pla Ma</t>
+          <t>Si Prachan</t>
         </is>
       </c>
       <c r="D744" t="n">
@@ -22014,16 +22014,16 @@
     </row>
     <row r="745">
       <c r="A745" t="n">
-        <v>7205</v>
+        <v>7206</v>
       </c>
       <c r="B745" t="inlineStr">
         <is>
-          <t>ศรีประจันต์</t>
+          <t>ดอนเจดีย์</t>
         </is>
       </c>
       <c r="C745" t="inlineStr">
         <is>
-          <t>Si Prachan</t>
+          <t>Don Chedi</t>
         </is>
       </c>
       <c r="D745" t="n">
@@ -22043,16 +22043,16 @@
     </row>
     <row r="746">
       <c r="A746" t="n">
-        <v>7206</v>
+        <v>7207</v>
       </c>
       <c r="B746" t="inlineStr">
         <is>
-          <t>ดอนเจดีย์</t>
+          <t>สองพี่น้อง</t>
         </is>
       </c>
       <c r="C746" t="inlineStr">
         <is>
-          <t>Don Chedi</t>
+          <t>Song Phi Nong</t>
         </is>
       </c>
       <c r="D746" t="n">
@@ -22072,16 +22072,16 @@
     </row>
     <row r="747">
       <c r="A747" t="n">
-        <v>7207</v>
+        <v>7208</v>
       </c>
       <c r="B747" t="inlineStr">
         <is>
-          <t>สองพี่น้อง</t>
+          <t>สามชุก</t>
         </is>
       </c>
       <c r="C747" t="inlineStr">
         <is>
-          <t>Song Phi Nong</t>
+          <t>Sam Chuk</t>
         </is>
       </c>
       <c r="D747" t="n">
@@ -22101,16 +22101,16 @@
     </row>
     <row r="748">
       <c r="A748" t="n">
-        <v>7208</v>
+        <v>7209</v>
       </c>
       <c r="B748" t="inlineStr">
         <is>
-          <t>สามชุก</t>
+          <t>อู่ทอง</t>
         </is>
       </c>
       <c r="C748" t="inlineStr">
         <is>
-          <t>Sam Chuk</t>
+          <t>U Thong</t>
         </is>
       </c>
       <c r="D748" t="n">
@@ -22130,16 +22130,16 @@
     </row>
     <row r="749">
       <c r="A749" t="n">
-        <v>7209</v>
+        <v>7210</v>
       </c>
       <c r="B749" t="inlineStr">
         <is>
-          <t>อู่ทอง</t>
+          <t>หนองหญ้าไซ</t>
         </is>
       </c>
       <c r="C749" t="inlineStr">
         <is>
-          <t>U Thong</t>
+          <t>Nong Ya Sai</t>
         </is>
       </c>
       <c r="D749" t="n">
@@ -22159,20 +22159,20 @@
     </row>
     <row r="750">
       <c r="A750" t="n">
-        <v>7210</v>
+        <v>7301</v>
       </c>
       <c r="B750" t="inlineStr">
         <is>
-          <t>หนองหญ้าไซ</t>
+          <t>เมืองนครปฐม</t>
         </is>
       </c>
       <c r="C750" t="inlineStr">
         <is>
-          <t>Nong Ya Sai</t>
+          <t>Mueang Nakhon Pathom</t>
         </is>
       </c>
       <c r="D750" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E750" t="inlineStr">
         <is>
@@ -22188,16 +22188,16 @@
     </row>
     <row r="751">
       <c r="A751" t="n">
-        <v>7301</v>
+        <v>7302</v>
       </c>
       <c r="B751" t="inlineStr">
         <is>
-          <t>เมืองนครปฐม</t>
+          <t>กำแพงแสน</t>
         </is>
       </c>
       <c r="C751" t="inlineStr">
         <is>
-          <t>Mueang Nakhon Pathom</t>
+          <t>Kamphaeng Saen</t>
         </is>
       </c>
       <c r="D751" t="n">
@@ -22217,16 +22217,16 @@
     </row>
     <row r="752">
       <c r="A752" t="n">
-        <v>7302</v>
+        <v>7303</v>
       </c>
       <c r="B752" t="inlineStr">
         <is>
-          <t>กำแพงแสน</t>
+          <t>นครชัยศรี</t>
         </is>
       </c>
       <c r="C752" t="inlineStr">
         <is>
-          <t>Kamphaeng Saen</t>
+          <t>Nakhon Chai Si</t>
         </is>
       </c>
       <c r="D752" t="n">
@@ -22246,16 +22246,16 @@
     </row>
     <row r="753">
       <c r="A753" t="n">
-        <v>7303</v>
+        <v>7304</v>
       </c>
       <c r="B753" t="inlineStr">
         <is>
-          <t>นครชัยศรี</t>
+          <t>ดอนตูม</t>
         </is>
       </c>
       <c r="C753" t="inlineStr">
         <is>
-          <t>Nakhon Chai Si</t>
+          <t>Don Tum</t>
         </is>
       </c>
       <c r="D753" t="n">
@@ -22275,16 +22275,16 @@
     </row>
     <row r="754">
       <c r="A754" t="n">
-        <v>7304</v>
+        <v>7305</v>
       </c>
       <c r="B754" t="inlineStr">
         <is>
-          <t>ดอนตูม</t>
+          <t>บางเลน</t>
         </is>
       </c>
       <c r="C754" t="inlineStr">
         <is>
-          <t>Don Tum</t>
+          <t>Bang Len</t>
         </is>
       </c>
       <c r="D754" t="n">
@@ -22304,16 +22304,16 @@
     </row>
     <row r="755">
       <c r="A755" t="n">
-        <v>7305</v>
+        <v>7306</v>
       </c>
       <c r="B755" t="inlineStr">
         <is>
-          <t>บางเลน</t>
+          <t>สามพราน</t>
         </is>
       </c>
       <c r="C755" t="inlineStr">
         <is>
-          <t>Bang Len</t>
+          <t>Sam Phran</t>
         </is>
       </c>
       <c r="D755" t="n">
@@ -22333,16 +22333,16 @@
     </row>
     <row r="756">
       <c r="A756" t="n">
-        <v>7306</v>
+        <v>7307</v>
       </c>
       <c r="B756" t="inlineStr">
         <is>
-          <t>สามพราน</t>
+          <t>พุทธมณฑล</t>
         </is>
       </c>
       <c r="C756" t="inlineStr">
         <is>
-          <t>Sam Phran</t>
+          <t>Phutthamonthon</t>
         </is>
       </c>
       <c r="D756" t="n">
@@ -22362,20 +22362,20 @@
     </row>
     <row r="757">
       <c r="A757" t="n">
-        <v>7307</v>
+        <v>7401</v>
       </c>
       <c r="B757" t="inlineStr">
         <is>
-          <t>พุทธมณฑล</t>
+          <t>เมืองสมุทรสาคร</t>
         </is>
       </c>
       <c r="C757" t="inlineStr">
         <is>
-          <t>Phutthamonthon</t>
+          <t>Mueang Samut Sakhon</t>
         </is>
       </c>
       <c r="D757" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E757" t="inlineStr">
         <is>
@@ -22391,16 +22391,16 @@
     </row>
     <row r="758">
       <c r="A758" t="n">
-        <v>7401</v>
+        <v>7402</v>
       </c>
       <c r="B758" t="inlineStr">
         <is>
-          <t>เมืองสมุทรสาคร</t>
+          <t>กระทุ่มแบน</t>
         </is>
       </c>
       <c r="C758" t="inlineStr">
         <is>
-          <t>Mueang Samut Sakhon</t>
+          <t>Krathum Baen</t>
         </is>
       </c>
       <c r="D758" t="n">
@@ -22420,16 +22420,16 @@
     </row>
     <row r="759">
       <c r="A759" t="n">
-        <v>7402</v>
+        <v>7403</v>
       </c>
       <c r="B759" t="inlineStr">
         <is>
-          <t>กระทุ่มแบน</t>
+          <t>บ้านแพ้ว</t>
         </is>
       </c>
       <c r="C759" t="inlineStr">
         <is>
-          <t>Krathum Baen</t>
+          <t>Ban Phaeo</t>
         </is>
       </c>
       <c r="D759" t="n">
@@ -22449,20 +22449,20 @@
     </row>
     <row r="760">
       <c r="A760" t="n">
-        <v>7403</v>
+        <v>7501</v>
       </c>
       <c r="B760" t="inlineStr">
         <is>
-          <t>บ้านแพ้ว</t>
+          <t>เมืองสมุทรสงคราม</t>
         </is>
       </c>
       <c r="C760" t="inlineStr">
         <is>
-          <t>Ban Phaeo</t>
+          <t>Mueang Samut Songkhram</t>
         </is>
       </c>
       <c r="D760" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E760" t="inlineStr">
         <is>
@@ -22478,16 +22478,16 @@
     </row>
     <row r="761">
       <c r="A761" t="n">
-        <v>7501</v>
+        <v>7502</v>
       </c>
       <c r="B761" t="inlineStr">
         <is>
-          <t>เมืองสมุทรสงคราม</t>
+          <t>บางคนที</t>
         </is>
       </c>
       <c r="C761" t="inlineStr">
         <is>
-          <t>Mueang Samut Songkhram</t>
+          <t>Bang Khonthi</t>
         </is>
       </c>
       <c r="D761" t="n">
@@ -22507,16 +22507,16 @@
     </row>
     <row r="762">
       <c r="A762" t="n">
-        <v>7502</v>
+        <v>7503</v>
       </c>
       <c r="B762" t="inlineStr">
         <is>
-          <t>บางคนที</t>
+          <t>อัมพวา</t>
         </is>
       </c>
       <c r="C762" t="inlineStr">
         <is>
-          <t>Bang Khonthi</t>
+          <t>Amphawa</t>
         </is>
       </c>
       <c r="D762" t="n">
@@ -22536,20 +22536,20 @@
     </row>
     <row r="763">
       <c r="A763" t="n">
-        <v>7503</v>
+        <v>7601</v>
       </c>
       <c r="B763" t="inlineStr">
         <is>
-          <t>อัมพวา</t>
+          <t>เมืองเพชรบุรี</t>
         </is>
       </c>
       <c r="C763" t="inlineStr">
         <is>
-          <t>Amphawa</t>
+          <t>Mueang Phetchaburi</t>
         </is>
       </c>
       <c r="D763" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E763" t="inlineStr">
         <is>
@@ -22565,16 +22565,16 @@
     </row>
     <row r="764">
       <c r="A764" t="n">
-        <v>7601</v>
+        <v>7602</v>
       </c>
       <c r="B764" t="inlineStr">
         <is>
-          <t>เมืองเพชรบุรี</t>
+          <t>เขาย้อย</t>
         </is>
       </c>
       <c r="C764" t="inlineStr">
         <is>
-          <t>Mueang Phetchaburi</t>
+          <t>Khao Yoi</t>
         </is>
       </c>
       <c r="D764" t="n">
@@ -22594,16 +22594,16 @@
     </row>
     <row r="765">
       <c r="A765" t="n">
-        <v>7602</v>
+        <v>7603</v>
       </c>
       <c r="B765" t="inlineStr">
         <is>
-          <t>เขาย้อย</t>
+          <t>หนองหญ้าปล้อง</t>
         </is>
       </c>
       <c r="C765" t="inlineStr">
         <is>
-          <t>Khao Yoi</t>
+          <t>Nong Ya Plong</t>
         </is>
       </c>
       <c r="D765" t="n">
@@ -22623,16 +22623,16 @@
     </row>
     <row r="766">
       <c r="A766" t="n">
-        <v>7603</v>
+        <v>7604</v>
       </c>
       <c r="B766" t="inlineStr">
         <is>
-          <t>หนองหญ้าปล้อง</t>
+          <t>ชะอำ</t>
         </is>
       </c>
       <c r="C766" t="inlineStr">
         <is>
-          <t>Nong Ya Plong</t>
+          <t>Cha-am</t>
         </is>
       </c>
       <c r="D766" t="n">
@@ -22652,16 +22652,16 @@
     </row>
     <row r="767">
       <c r="A767" t="n">
-        <v>7604</v>
+        <v>7605</v>
       </c>
       <c r="B767" t="inlineStr">
         <is>
-          <t>ชะอำ</t>
+          <t>ท่ายาง</t>
         </is>
       </c>
       <c r="C767" t="inlineStr">
         <is>
-          <t>Cha-am</t>
+          <t>Tha Yang</t>
         </is>
       </c>
       <c r="D767" t="n">
@@ -22681,16 +22681,16 @@
     </row>
     <row r="768">
       <c r="A768" t="n">
-        <v>7605</v>
+        <v>7606</v>
       </c>
       <c r="B768" t="inlineStr">
         <is>
-          <t>ท่ายาง</t>
+          <t>บ้านลาด</t>
         </is>
       </c>
       <c r="C768" t="inlineStr">
         <is>
-          <t>Tha Yang</t>
+          <t>Ban Lat</t>
         </is>
       </c>
       <c r="D768" t="n">
@@ -22710,16 +22710,16 @@
     </row>
     <row r="769">
       <c r="A769" t="n">
-        <v>7606</v>
+        <v>7607</v>
       </c>
       <c r="B769" t="inlineStr">
         <is>
-          <t>บ้านลาด</t>
+          <t>บ้านแหลม</t>
         </is>
       </c>
       <c r="C769" t="inlineStr">
         <is>
-          <t>Ban Lat</t>
+          <t>Ban Laem</t>
         </is>
       </c>
       <c r="D769" t="n">
@@ -22739,16 +22739,16 @@
     </row>
     <row r="770">
       <c r="A770" t="n">
-        <v>7607</v>
+        <v>7608</v>
       </c>
       <c r="B770" t="inlineStr">
         <is>
-          <t>บ้านแหลม</t>
+          <t>แก่งกระจาน</t>
         </is>
       </c>
       <c r="C770" t="inlineStr">
         <is>
-          <t>Ban Laem</t>
+          <t>Kaeng Krachan</t>
         </is>
       </c>
       <c r="D770" t="n">
@@ -22768,20 +22768,20 @@
     </row>
     <row r="771">
       <c r="A771" t="n">
-        <v>7608</v>
+        <v>7701</v>
       </c>
       <c r="B771" t="inlineStr">
         <is>
-          <t>แก่งกระจาน</t>
+          <t>เมืองประจวบคีรีขันธ์</t>
         </is>
       </c>
       <c r="C771" t="inlineStr">
         <is>
-          <t>Kaeng Krachan</t>
+          <t>Mueang Prachuap Khiri Khan</t>
         </is>
       </c>
       <c r="D771" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E771" t="inlineStr">
         <is>
@@ -22797,16 +22797,16 @@
     </row>
     <row r="772">
       <c r="A772" t="n">
-        <v>7701</v>
+        <v>7702</v>
       </c>
       <c r="B772" t="inlineStr">
         <is>
-          <t>เมืองประจวบคีรีขันธ์</t>
+          <t>กุยบุรี</t>
         </is>
       </c>
       <c r="C772" t="inlineStr">
         <is>
-          <t>Mueang Prachuap Khiri Khan</t>
+          <t>Kui Buri</t>
         </is>
       </c>
       <c r="D772" t="n">
@@ -22826,16 +22826,16 @@
     </row>
     <row r="773">
       <c r="A773" t="n">
-        <v>7702</v>
+        <v>7703</v>
       </c>
       <c r="B773" t="inlineStr">
         <is>
-          <t>กุยบุรี</t>
+          <t>ทับสะแก</t>
         </is>
       </c>
       <c r="C773" t="inlineStr">
         <is>
-          <t>Kui Buri</t>
+          <t>Thap Sakae</t>
         </is>
       </c>
       <c r="D773" t="n">
@@ -22855,16 +22855,16 @@
     </row>
     <row r="774">
       <c r="A774" t="n">
-        <v>7703</v>
+        <v>7704</v>
       </c>
       <c r="B774" t="inlineStr">
         <is>
-          <t>ทับสะแก</t>
+          <t>บางสะพาน</t>
         </is>
       </c>
       <c r="C774" t="inlineStr">
         <is>
-          <t>Thap Sakae</t>
+          <t>Bang Saphan</t>
         </is>
       </c>
       <c r="D774" t="n">
@@ -22884,16 +22884,16 @@
     </row>
     <row r="775">
       <c r="A775" t="n">
-        <v>7704</v>
+        <v>7705</v>
       </c>
       <c r="B775" t="inlineStr">
         <is>
-          <t>บางสะพาน</t>
+          <t>บางสะพานน้อย</t>
         </is>
       </c>
       <c r="C775" t="inlineStr">
         <is>
-          <t>Bang Saphan</t>
+          <t>Bang Saphan Noi</t>
         </is>
       </c>
       <c r="D775" t="n">
@@ -22913,16 +22913,16 @@
     </row>
     <row r="776">
       <c r="A776" t="n">
-        <v>7705</v>
+        <v>7706</v>
       </c>
       <c r="B776" t="inlineStr">
         <is>
-          <t>บางสะพานน้อย</t>
+          <t>ปราณบุรี</t>
         </is>
       </c>
       <c r="C776" t="inlineStr">
         <is>
-          <t>Bang Saphan Noi</t>
+          <t>Pran Buri</t>
         </is>
       </c>
       <c r="D776" t="n">
@@ -22942,16 +22942,16 @@
     </row>
     <row r="777">
       <c r="A777" t="n">
-        <v>7706</v>
+        <v>7707</v>
       </c>
       <c r="B777" t="inlineStr">
         <is>
-          <t>ปราณบุรี</t>
+          <t>หัวหิน</t>
         </is>
       </c>
       <c r="C777" t="inlineStr">
         <is>
-          <t>Pran Buri</t>
+          <t>Hua Hin</t>
         </is>
       </c>
       <c r="D777" t="n">
@@ -22971,16 +22971,16 @@
     </row>
     <row r="778">
       <c r="A778" t="n">
-        <v>7707</v>
+        <v>7708</v>
       </c>
       <c r="B778" t="inlineStr">
         <is>
-          <t>หัวหิน</t>
+          <t>สามร้อยยอด</t>
         </is>
       </c>
       <c r="C778" t="inlineStr">
         <is>
-          <t>Hua Hin</t>
+          <t>Sam Roi Yot</t>
         </is>
       </c>
       <c r="D778" t="n">
@@ -23000,20 +23000,20 @@
     </row>
     <row r="779">
       <c r="A779" t="n">
-        <v>7708</v>
+        <v>8001</v>
       </c>
       <c r="B779" t="inlineStr">
         <is>
-          <t>สามร้อยยอด</t>
+          <t>เมืองนครศรีธรรมราช</t>
         </is>
       </c>
       <c r="C779" t="inlineStr">
         <is>
-          <t>Sam Roi Yot</t>
+          <t>Mueang Nakhon Si Thammarat</t>
         </is>
       </c>
       <c r="D779" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E779" t="inlineStr">
         <is>
@@ -23029,16 +23029,16 @@
     </row>
     <row r="780">
       <c r="A780" t="n">
-        <v>8001</v>
+        <v>8002</v>
       </c>
       <c r="B780" t="inlineStr">
         <is>
-          <t>เมืองนครศรีธรรมราช</t>
+          <t>พรหมคีรี</t>
         </is>
       </c>
       <c r="C780" t="inlineStr">
         <is>
-          <t>Mueang Nakhon Si Thammarat</t>
+          <t>Phrom Khiri</t>
         </is>
       </c>
       <c r="D780" t="n">
@@ -23058,16 +23058,16 @@
     </row>
     <row r="781">
       <c r="A781" t="n">
-        <v>8002</v>
+        <v>8003</v>
       </c>
       <c r="B781" t="inlineStr">
         <is>
-          <t>พรหมคีรี</t>
+          <t>ลานสกา</t>
         </is>
       </c>
       <c r="C781" t="inlineStr">
         <is>
-          <t>Phrom Khiri</t>
+          <t>Lan Saka</t>
         </is>
       </c>
       <c r="D781" t="n">
@@ -23087,16 +23087,16 @@
     </row>
     <row r="782">
       <c r="A782" t="n">
-        <v>8003</v>
+        <v>8004</v>
       </c>
       <c r="B782" t="inlineStr">
         <is>
-          <t>ลานสกา</t>
+          <t>ฉวาง</t>
         </is>
       </c>
       <c r="C782" t="inlineStr">
         <is>
-          <t>Lan Saka</t>
+          <t>Chawang</t>
         </is>
       </c>
       <c r="D782" t="n">
@@ -23116,16 +23116,16 @@
     </row>
     <row r="783">
       <c r="A783" t="n">
-        <v>8004</v>
+        <v>8005</v>
       </c>
       <c r="B783" t="inlineStr">
         <is>
-          <t>ฉวาง</t>
+          <t>พิปูน</t>
         </is>
       </c>
       <c r="C783" t="inlineStr">
         <is>
-          <t>Chawang</t>
+          <t>Phipun</t>
         </is>
       </c>
       <c r="D783" t="n">
@@ -23145,16 +23145,16 @@
     </row>
     <row r="784">
       <c r="A784" t="n">
-        <v>8005</v>
+        <v>8006</v>
       </c>
       <c r="B784" t="inlineStr">
         <is>
-          <t>พิปูน</t>
+          <t>เชียรใหญ่</t>
         </is>
       </c>
       <c r="C784" t="inlineStr">
         <is>
-          <t>Phipun</t>
+          <t>Chian Yai</t>
         </is>
       </c>
       <c r="D784" t="n">
@@ -23174,16 +23174,16 @@
     </row>
     <row r="785">
       <c r="A785" t="n">
-        <v>8006</v>
+        <v>8007</v>
       </c>
       <c r="B785" t="inlineStr">
         <is>
-          <t>เชียรใหญ่</t>
+          <t>ชะอวด</t>
         </is>
       </c>
       <c r="C785" t="inlineStr">
         <is>
-          <t>Chian Yai</t>
+          <t>Cha-uat</t>
         </is>
       </c>
       <c r="D785" t="n">
@@ -23203,16 +23203,16 @@
     </row>
     <row r="786">
       <c r="A786" t="n">
-        <v>8007</v>
+        <v>8008</v>
       </c>
       <c r="B786" t="inlineStr">
         <is>
-          <t>ชะอวด</t>
+          <t>ท่าศาลา</t>
         </is>
       </c>
       <c r="C786" t="inlineStr">
         <is>
-          <t>Cha-uat</t>
+          <t>Tha Sala</t>
         </is>
       </c>
       <c r="D786" t="n">
@@ -23232,16 +23232,16 @@
     </row>
     <row r="787">
       <c r="A787" t="n">
-        <v>8008</v>
+        <v>8009</v>
       </c>
       <c r="B787" t="inlineStr">
         <is>
-          <t>ท่าศาลา</t>
+          <t>ทุ่งสง</t>
         </is>
       </c>
       <c r="C787" t="inlineStr">
         <is>
-          <t>Tha Sala</t>
+          <t>Thung Song</t>
         </is>
       </c>
       <c r="D787" t="n">
@@ -23261,16 +23261,16 @@
     </row>
     <row r="788">
       <c r="A788" t="n">
-        <v>8009</v>
+        <v>8010</v>
       </c>
       <c r="B788" t="inlineStr">
         <is>
-          <t>ทุ่งสง</t>
+          <t>นาบอน</t>
         </is>
       </c>
       <c r="C788" t="inlineStr">
         <is>
-          <t>Thung Song</t>
+          <t>Na Bon</t>
         </is>
       </c>
       <c r="D788" t="n">
@@ -23290,16 +23290,16 @@
     </row>
     <row r="789">
       <c r="A789" t="n">
-        <v>8010</v>
+        <v>8011</v>
       </c>
       <c r="B789" t="inlineStr">
         <is>
-          <t>นาบอน</t>
+          <t>ทุ่งใหญ่</t>
         </is>
       </c>
       <c r="C789" t="inlineStr">
         <is>
-          <t>Na Bon</t>
+          <t>Thung Yai</t>
         </is>
       </c>
       <c r="D789" t="n">
@@ -23319,16 +23319,16 @@
     </row>
     <row r="790">
       <c r="A790" t="n">
-        <v>8011</v>
+        <v>8012</v>
       </c>
       <c r="B790" t="inlineStr">
         <is>
-          <t>ทุ่งใหญ่</t>
+          <t>ปากพนัง</t>
         </is>
       </c>
       <c r="C790" t="inlineStr">
         <is>
-          <t>Thung Yai</t>
+          <t>Pak Phanang</t>
         </is>
       </c>
       <c r="D790" t="n">
@@ -23348,16 +23348,16 @@
     </row>
     <row r="791">
       <c r="A791" t="n">
-        <v>8012</v>
+        <v>8013</v>
       </c>
       <c r="B791" t="inlineStr">
         <is>
-          <t>ปากพนัง</t>
+          <t>ร่อนพิบูลย์</t>
         </is>
       </c>
       <c r="C791" t="inlineStr">
         <is>
-          <t>Pak Phanang</t>
+          <t>Ron Phibun</t>
         </is>
       </c>
       <c r="D791" t="n">
@@ -23377,16 +23377,16 @@
     </row>
     <row r="792">
       <c r="A792" t="n">
-        <v>8013</v>
+        <v>8014</v>
       </c>
       <c r="B792" t="inlineStr">
         <is>
-          <t>ร่อนพิบูลย์</t>
+          <t>สิชล</t>
         </is>
       </c>
       <c r="C792" t="inlineStr">
         <is>
-          <t>Ron Phibun</t>
+          <t>Sichon</t>
         </is>
       </c>
       <c r="D792" t="n">
@@ -23406,16 +23406,16 @@
     </row>
     <row r="793">
       <c r="A793" t="n">
-        <v>8014</v>
+        <v>8015</v>
       </c>
       <c r="B793" t="inlineStr">
         <is>
-          <t>สิชล</t>
+          <t>ขนอม</t>
         </is>
       </c>
       <c r="C793" t="inlineStr">
         <is>
-          <t>Sichon</t>
+          <t>Khanom</t>
         </is>
       </c>
       <c r="D793" t="n">
@@ -23435,16 +23435,16 @@
     </row>
     <row r="794">
       <c r="A794" t="n">
-        <v>8015</v>
+        <v>8016</v>
       </c>
       <c r="B794" t="inlineStr">
         <is>
-          <t>ขนอม</t>
+          <t>หัวไทร</t>
         </is>
       </c>
       <c r="C794" t="inlineStr">
         <is>
-          <t>Khanom</t>
+          <t>Hua Sai</t>
         </is>
       </c>
       <c r="D794" t="n">
@@ -23464,16 +23464,16 @@
     </row>
     <row r="795">
       <c r="A795" t="n">
-        <v>8016</v>
+        <v>8017</v>
       </c>
       <c r="B795" t="inlineStr">
         <is>
-          <t>หัวไทร</t>
+          <t>บางขัน</t>
         </is>
       </c>
       <c r="C795" t="inlineStr">
         <is>
-          <t>Hua Sai</t>
+          <t>Bang Khan</t>
         </is>
       </c>
       <c r="D795" t="n">
@@ -23493,16 +23493,16 @@
     </row>
     <row r="796">
       <c r="A796" t="n">
-        <v>8017</v>
+        <v>8018</v>
       </c>
       <c r="B796" t="inlineStr">
         <is>
-          <t>บางขัน</t>
+          <t>ถ้ำพรรณรา</t>
         </is>
       </c>
       <c r="C796" t="inlineStr">
         <is>
-          <t>Bang Khan</t>
+          <t>Tham Phannara</t>
         </is>
       </c>
       <c r="D796" t="n">
@@ -23522,16 +23522,16 @@
     </row>
     <row r="797">
       <c r="A797" t="n">
-        <v>8018</v>
+        <v>8019</v>
       </c>
       <c r="B797" t="inlineStr">
         <is>
-          <t>ถ้ำพรรณรา</t>
+          <t>จุฬาภรณ์</t>
         </is>
       </c>
       <c r="C797" t="inlineStr">
         <is>
-          <t>Tham Phannara</t>
+          <t>Chulabhorn</t>
         </is>
       </c>
       <c r="D797" t="n">
@@ -23551,16 +23551,16 @@
     </row>
     <row r="798">
       <c r="A798" t="n">
-        <v>8019</v>
+        <v>8020</v>
       </c>
       <c r="B798" t="inlineStr">
         <is>
-          <t>จุฬาภรณ์</t>
+          <t>พระพรหม</t>
         </is>
       </c>
       <c r="C798" t="inlineStr">
         <is>
-          <t>Chulabhorn</t>
+          <t>Phra Phrom</t>
         </is>
       </c>
       <c r="D798" t="n">
@@ -23580,16 +23580,16 @@
     </row>
     <row r="799">
       <c r="A799" t="n">
-        <v>8020</v>
+        <v>8021</v>
       </c>
       <c r="B799" t="inlineStr">
         <is>
-          <t>พระพรหม</t>
+          <t>นบพิตำ</t>
         </is>
       </c>
       <c r="C799" t="inlineStr">
         <is>
-          <t>Phra Phrom</t>
+          <t>Nopphitam</t>
         </is>
       </c>
       <c r="D799" t="n">
@@ -23609,16 +23609,16 @@
     </row>
     <row r="800">
       <c r="A800" t="n">
-        <v>8021</v>
+        <v>8022</v>
       </c>
       <c r="B800" t="inlineStr">
         <is>
-          <t>นบพิตำ</t>
+          <t>ช้างกลาง</t>
         </is>
       </c>
       <c r="C800" t="inlineStr">
         <is>
-          <t>Nopphitam</t>
+          <t>Chang Klang</t>
         </is>
       </c>
       <c r="D800" t="n">
@@ -23638,16 +23638,16 @@
     </row>
     <row r="801">
       <c r="A801" t="n">
-        <v>8022</v>
+        <v>8023</v>
       </c>
       <c r="B801" t="inlineStr">
         <is>
-          <t>ช้างกลาง</t>
+          <t>เฉลิมพระเกียรติ</t>
         </is>
       </c>
       <c r="C801" t="inlineStr">
         <is>
-          <t>Chang Klang</t>
+          <t>Chaloem Phra Kiat</t>
         </is>
       </c>
       <c r="D801" t="n">
@@ -23667,20 +23667,20 @@
     </row>
     <row r="802">
       <c r="A802" t="n">
-        <v>8023</v>
+        <v>8101</v>
       </c>
       <c r="B802" t="inlineStr">
         <is>
-          <t>เฉลิมพระเกียรติ</t>
+          <t>เมืองกระบี่</t>
         </is>
       </c>
       <c r="C802" t="inlineStr">
         <is>
-          <t>Chaloem Phra Kiat</t>
+          <t>Mueang Krabi</t>
         </is>
       </c>
       <c r="D802" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E802" t="inlineStr">
         <is>
@@ -23696,16 +23696,16 @@
     </row>
     <row r="803">
       <c r="A803" t="n">
-        <v>8101</v>
+        <v>8102</v>
       </c>
       <c r="B803" t="inlineStr">
         <is>
-          <t>เมืองกระบี่</t>
+          <t>เขาพนม</t>
         </is>
       </c>
       <c r="C803" t="inlineStr">
         <is>
-          <t>Mueang Krabi</t>
+          <t>Khao Phanom</t>
         </is>
       </c>
       <c r="D803" t="n">
@@ -23725,16 +23725,16 @@
     </row>
     <row r="804">
       <c r="A804" t="n">
-        <v>8102</v>
+        <v>8103</v>
       </c>
       <c r="B804" t="inlineStr">
         <is>
-          <t>เขาพนม</t>
+          <t>เกาะลันตา</t>
         </is>
       </c>
       <c r="C804" t="inlineStr">
         <is>
-          <t>Khao Phanom</t>
+          <t>Ko Lanta</t>
         </is>
       </c>
       <c r="D804" t="n">
@@ -23754,16 +23754,16 @@
     </row>
     <row r="805">
       <c r="A805" t="n">
-        <v>8103</v>
+        <v>8104</v>
       </c>
       <c r="B805" t="inlineStr">
         <is>
-          <t>เกาะลันตา</t>
+          <t>คลองท่อม</t>
         </is>
       </c>
       <c r="C805" t="inlineStr">
         <is>
-          <t>Ko Lanta</t>
+          <t>Khlong Thom</t>
         </is>
       </c>
       <c r="D805" t="n">
@@ -23783,16 +23783,16 @@
     </row>
     <row r="806">
       <c r="A806" t="n">
-        <v>8104</v>
+        <v>8105</v>
       </c>
       <c r="B806" t="inlineStr">
         <is>
-          <t>คลองท่อม</t>
+          <t>อ่าวลึก</t>
         </is>
       </c>
       <c r="C806" t="inlineStr">
         <is>
-          <t>Khlong Thom</t>
+          <t>Ao Luek</t>
         </is>
       </c>
       <c r="D806" t="n">
@@ -23812,16 +23812,16 @@
     </row>
     <row r="807">
       <c r="A807" t="n">
-        <v>8105</v>
+        <v>8106</v>
       </c>
       <c r="B807" t="inlineStr">
         <is>
-          <t>อ่าวลึก</t>
+          <t>ปลายพระยา</t>
         </is>
       </c>
       <c r="C807" t="inlineStr">
         <is>
-          <t>Ao Luek</t>
+          <t>Plai Phraya</t>
         </is>
       </c>
       <c r="D807" t="n">
@@ -23841,16 +23841,16 @@
     </row>
     <row r="808">
       <c r="A808" t="n">
-        <v>8106</v>
+        <v>8107</v>
       </c>
       <c r="B808" t="inlineStr">
         <is>
-          <t>ปลายพระยา</t>
+          <t>ลำทับ</t>
         </is>
       </c>
       <c r="C808" t="inlineStr">
         <is>
-          <t>Plai Phraya</t>
+          <t>Lam Thap</t>
         </is>
       </c>
       <c r="D808" t="n">
@@ -23870,16 +23870,16 @@
     </row>
     <row r="809">
       <c r="A809" t="n">
-        <v>8107</v>
+        <v>8108</v>
       </c>
       <c r="B809" t="inlineStr">
         <is>
-          <t>ลำทับ</t>
+          <t>เหนือคลอง</t>
         </is>
       </c>
       <c r="C809" t="inlineStr">
         <is>
-          <t>Lam Thap</t>
+          <t>Nuea Khlong</t>
         </is>
       </c>
       <c r="D809" t="n">
@@ -23899,20 +23899,20 @@
     </row>
     <row r="810">
       <c r="A810" t="n">
-        <v>8108</v>
+        <v>8201</v>
       </c>
       <c r="B810" t="inlineStr">
         <is>
-          <t>เหนือคลอง</t>
+          <t>เมืองพังงา</t>
         </is>
       </c>
       <c r="C810" t="inlineStr">
         <is>
-          <t>Nuea Khlong</t>
+          <t>Mueang Phang-nga</t>
         </is>
       </c>
       <c r="D810" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E810" t="inlineStr">
         <is>
@@ -23928,16 +23928,16 @@
     </row>
     <row r="811">
       <c r="A811" t="n">
-        <v>8201</v>
+        <v>8202</v>
       </c>
       <c r="B811" t="inlineStr">
         <is>
-          <t>เมืองพังงา</t>
+          <t>เกาะยาว</t>
         </is>
       </c>
       <c r="C811" t="inlineStr">
         <is>
-          <t>Mueang Phang-nga</t>
+          <t>Ko Yao</t>
         </is>
       </c>
       <c r="D811" t="n">
@@ -23957,16 +23957,16 @@
     </row>
     <row r="812">
       <c r="A812" t="n">
-        <v>8202</v>
+        <v>8203</v>
       </c>
       <c r="B812" t="inlineStr">
         <is>
-          <t>เกาะยาว</t>
+          <t>กะปง</t>
         </is>
       </c>
       <c r="C812" t="inlineStr">
         <is>
-          <t>Ko Yao</t>
+          <t>Kapong</t>
         </is>
       </c>
       <c r="D812" t="n">
@@ -23986,16 +23986,16 @@
     </row>
     <row r="813">
       <c r="A813" t="n">
-        <v>8203</v>
+        <v>8204</v>
       </c>
       <c r="B813" t="inlineStr">
         <is>
-          <t>กะปง</t>
+          <t>ตะกั่วทุ่ง</t>
         </is>
       </c>
       <c r="C813" t="inlineStr">
         <is>
-          <t>Kapong</t>
+          <t>Takua Thung</t>
         </is>
       </c>
       <c r="D813" t="n">
@@ -24015,16 +24015,16 @@
     </row>
     <row r="814">
       <c r="A814" t="n">
-        <v>8204</v>
+        <v>8205</v>
       </c>
       <c r="B814" t="inlineStr">
         <is>
-          <t>ตะกั่วทุ่ง</t>
+          <t>ตะกั่วป่า</t>
         </is>
       </c>
       <c r="C814" t="inlineStr">
         <is>
-          <t>Takua Thung</t>
+          <t>Takua Pa</t>
         </is>
       </c>
       <c r="D814" t="n">
@@ -24044,16 +24044,16 @@
     </row>
     <row r="815">
       <c r="A815" t="n">
-        <v>8205</v>
+        <v>8206</v>
       </c>
       <c r="B815" t="inlineStr">
         <is>
-          <t>ตะกั่วป่า</t>
+          <t>คุระบุรี</t>
         </is>
       </c>
       <c r="C815" t="inlineStr">
         <is>
-          <t>Takua Pa</t>
+          <t>Khura Buri</t>
         </is>
       </c>
       <c r="D815" t="n">
@@ -24073,16 +24073,16 @@
     </row>
     <row r="816">
       <c r="A816" t="n">
-        <v>8206</v>
+        <v>8207</v>
       </c>
       <c r="B816" t="inlineStr">
         <is>
-          <t>คุระบุรี</t>
+          <t>ทับปุด</t>
         </is>
       </c>
       <c r="C816" t="inlineStr">
         <is>
-          <t>Khura Buri</t>
+          <t>Thap Put</t>
         </is>
       </c>
       <c r="D816" t="n">
@@ -24102,16 +24102,16 @@
     </row>
     <row r="817">
       <c r="A817" t="n">
-        <v>8207</v>
+        <v>8208</v>
       </c>
       <c r="B817" t="inlineStr">
         <is>
-          <t>ทับปุด</t>
+          <t>ท้ายเหมือง</t>
         </is>
       </c>
       <c r="C817" t="inlineStr">
         <is>
-          <t>Thap Put</t>
+          <t>Thai Mueang</t>
         </is>
       </c>
       <c r="D817" t="n">
@@ -24131,20 +24131,20 @@
     </row>
     <row r="818">
       <c r="A818" t="n">
-        <v>8208</v>
+        <v>8301</v>
       </c>
       <c r="B818" t="inlineStr">
         <is>
-          <t>ท้ายเหมือง</t>
+          <t>เมืองภูเก็ต</t>
         </is>
       </c>
       <c r="C818" t="inlineStr">
         <is>
-          <t>Thai Mueang</t>
+          <t>Mueang Phuket</t>
         </is>
       </c>
       <c r="D818" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E818" t="inlineStr">
         <is>
@@ -24160,16 +24160,16 @@
     </row>
     <row r="819">
       <c r="A819" t="n">
-        <v>8301</v>
+        <v>8302</v>
       </c>
       <c r="B819" t="inlineStr">
         <is>
-          <t>เมืองภูเก็ต</t>
+          <t>กะทู้</t>
         </is>
       </c>
       <c r="C819" t="inlineStr">
         <is>
-          <t>Mueang Phuket</t>
+          <t>Kathu</t>
         </is>
       </c>
       <c r="D819" t="n">
@@ -24189,16 +24189,16 @@
     </row>
     <row r="820">
       <c r="A820" t="n">
-        <v>8302</v>
+        <v>8303</v>
       </c>
       <c r="B820" t="inlineStr">
         <is>
-          <t>กะทู้</t>
+          <t>ถลาง</t>
         </is>
       </c>
       <c r="C820" t="inlineStr">
         <is>
-          <t>Kathu</t>
+          <t>Thalang</t>
         </is>
       </c>
       <c r="D820" t="n">
@@ -24218,20 +24218,20 @@
     </row>
     <row r="821">
       <c r="A821" t="n">
-        <v>8303</v>
+        <v>8401</v>
       </c>
       <c r="B821" t="inlineStr">
         <is>
-          <t>ถลาง</t>
+          <t>เมืองสุราษฎร์ธานี</t>
         </is>
       </c>
       <c r="C821" t="inlineStr">
         <is>
-          <t>Thalang</t>
+          <t>Mueang Surat Thani</t>
         </is>
       </c>
       <c r="D821" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E821" t="inlineStr">
         <is>
@@ -24247,16 +24247,16 @@
     </row>
     <row r="822">
       <c r="A822" t="n">
-        <v>8401</v>
+        <v>8402</v>
       </c>
       <c r="B822" t="inlineStr">
         <is>
-          <t>เมืองสุราษฎร์ธานี</t>
+          <t>กาญจนดิษฐ์</t>
         </is>
       </c>
       <c r="C822" t="inlineStr">
         <is>
-          <t>Mueang Surat Thani</t>
+          <t>Kanchanadit</t>
         </is>
       </c>
       <c r="D822" t="n">
@@ -24276,16 +24276,16 @@
     </row>
     <row r="823">
       <c r="A823" t="n">
-        <v>8402</v>
+        <v>8403</v>
       </c>
       <c r="B823" t="inlineStr">
         <is>
-          <t>กาญจนดิษฐ์</t>
+          <t>ดอนสัก</t>
         </is>
       </c>
       <c r="C823" t="inlineStr">
         <is>
-          <t>Kanchanadit</t>
+          <t>Don Sak</t>
         </is>
       </c>
       <c r="D823" t="n">
@@ -24305,16 +24305,16 @@
     </row>
     <row r="824">
       <c r="A824" t="n">
-        <v>8403</v>
+        <v>8404</v>
       </c>
       <c r="B824" t="inlineStr">
         <is>
-          <t>ดอนสัก</t>
+          <t>เกาะสมุย</t>
         </is>
       </c>
       <c r="C824" t="inlineStr">
         <is>
-          <t>Don Sak</t>
+          <t>Ko Samui</t>
         </is>
       </c>
       <c r="D824" t="n">
@@ -24334,16 +24334,16 @@
     </row>
     <row r="825">
       <c r="A825" t="n">
-        <v>8404</v>
+        <v>8405</v>
       </c>
       <c r="B825" t="inlineStr">
         <is>
-          <t>เกาะสมุย</t>
+          <t>เกาะพะงัน</t>
         </is>
       </c>
       <c r="C825" t="inlineStr">
         <is>
-          <t>Ko Samui</t>
+          <t>Ko Pha-ngan</t>
         </is>
       </c>
       <c r="D825" t="n">
@@ -24363,16 +24363,16 @@
     </row>
     <row r="826">
       <c r="A826" t="n">
-        <v>8405</v>
+        <v>8406</v>
       </c>
       <c r="B826" t="inlineStr">
         <is>
-          <t>เกาะพะงัน</t>
+          <t>ไชยา</t>
         </is>
       </c>
       <c r="C826" t="inlineStr">
         <is>
-          <t>Ko Pha-ngan</t>
+          <t>Chaiya</t>
         </is>
       </c>
       <c r="D826" t="n">
@@ -24392,16 +24392,16 @@
     </row>
     <row r="827">
       <c r="A827" t="n">
-        <v>8406</v>
+        <v>8407</v>
       </c>
       <c r="B827" t="inlineStr">
         <is>
-          <t>ไชยา</t>
+          <t>ท่าชนะ</t>
         </is>
       </c>
       <c r="C827" t="inlineStr">
         <is>
-          <t>Chaiya</t>
+          <t>Tha Chana</t>
         </is>
       </c>
       <c r="D827" t="n">
@@ -24421,16 +24421,16 @@
     </row>
     <row r="828">
       <c r="A828" t="n">
-        <v>8407</v>
+        <v>8408</v>
       </c>
       <c r="B828" t="inlineStr">
         <is>
-          <t>ท่าชนะ</t>
+          <t>คีรีรัฐนิคม</t>
         </is>
       </c>
       <c r="C828" t="inlineStr">
         <is>
-          <t>Tha Chana</t>
+          <t>Khiri Rat Nikhom</t>
         </is>
       </c>
       <c r="D828" t="n">
@@ -24450,16 +24450,16 @@
     </row>
     <row r="829">
       <c r="A829" t="n">
-        <v>8408</v>
+        <v>8409</v>
       </c>
       <c r="B829" t="inlineStr">
         <is>
-          <t>คีรีรัฐนิคม</t>
+          <t>บ้านตาขุน</t>
         </is>
       </c>
       <c r="C829" t="inlineStr">
         <is>
-          <t>Khiri Rat Nikhom</t>
+          <t>Ban Ta Khun</t>
         </is>
       </c>
       <c r="D829" t="n">
@@ -24479,16 +24479,16 @@
     </row>
     <row r="830">
       <c r="A830" t="n">
-        <v>8409</v>
+        <v>8410</v>
       </c>
       <c r="B830" t="inlineStr">
         <is>
-          <t>บ้านตาขุน</t>
+          <t>พนม</t>
         </is>
       </c>
       <c r="C830" t="inlineStr">
         <is>
-          <t>Ban Ta Khun</t>
+          <t>Phanom</t>
         </is>
       </c>
       <c r="D830" t="n">
@@ -24508,16 +24508,16 @@
     </row>
     <row r="831">
       <c r="A831" t="n">
-        <v>8410</v>
+        <v>8411</v>
       </c>
       <c r="B831" t="inlineStr">
         <is>
-          <t>พนม</t>
+          <t>ท่าฉาง</t>
         </is>
       </c>
       <c r="C831" t="inlineStr">
         <is>
-          <t>Phanom</t>
+          <t>Tha Chang</t>
         </is>
       </c>
       <c r="D831" t="n">
@@ -24537,16 +24537,16 @@
     </row>
     <row r="832">
       <c r="A832" t="n">
-        <v>8411</v>
+        <v>8412</v>
       </c>
       <c r="B832" t="inlineStr">
         <is>
-          <t>ท่าฉาง</t>
+          <t>บ้านนาสาร</t>
         </is>
       </c>
       <c r="C832" t="inlineStr">
         <is>
-          <t>Tha Chang</t>
+          <t>Ban Na San</t>
         </is>
       </c>
       <c r="D832" t="n">
@@ -24566,16 +24566,16 @@
     </row>
     <row r="833">
       <c r="A833" t="n">
-        <v>8412</v>
+        <v>8413</v>
       </c>
       <c r="B833" t="inlineStr">
         <is>
-          <t>บ้านนาสาร</t>
+          <t>บ้านนาเดิม</t>
         </is>
       </c>
       <c r="C833" t="inlineStr">
         <is>
-          <t>Ban Na San</t>
+          <t>Ban Na Doem</t>
         </is>
       </c>
       <c r="D833" t="n">
@@ -24595,16 +24595,16 @@
     </row>
     <row r="834">
       <c r="A834" t="n">
-        <v>8413</v>
+        <v>8414</v>
       </c>
       <c r="B834" t="inlineStr">
         <is>
-          <t>บ้านนาเดิม</t>
+          <t>เคียนซา</t>
         </is>
       </c>
       <c r="C834" t="inlineStr">
         <is>
-          <t>Ban Na Doem</t>
+          <t>Khian Sa</t>
         </is>
       </c>
       <c r="D834" t="n">
@@ -24624,16 +24624,16 @@
     </row>
     <row r="835">
       <c r="A835" t="n">
-        <v>8414</v>
+        <v>8415</v>
       </c>
       <c r="B835" t="inlineStr">
         <is>
-          <t>เคียนซา</t>
+          <t>เวียงสระ</t>
         </is>
       </c>
       <c r="C835" t="inlineStr">
         <is>
-          <t>Khian Sa</t>
+          <t>Wiang Sa</t>
         </is>
       </c>
       <c r="D835" t="n">
@@ -24653,16 +24653,16 @@
     </row>
     <row r="836">
       <c r="A836" t="n">
-        <v>8415</v>
+        <v>8416</v>
       </c>
       <c r="B836" t="inlineStr">
         <is>
-          <t>เวียงสระ</t>
+          <t>พระแสง</t>
         </is>
       </c>
       <c r="C836" t="inlineStr">
         <is>
-          <t>Wiang Sa</t>
+          <t>Phrasaeng</t>
         </is>
       </c>
       <c r="D836" t="n">
@@ -24682,16 +24682,16 @@
     </row>
     <row r="837">
       <c r="A837" t="n">
-        <v>8416</v>
+        <v>8417</v>
       </c>
       <c r="B837" t="inlineStr">
         <is>
-          <t>พระแสง</t>
+          <t>พุนพิน</t>
         </is>
       </c>
       <c r="C837" t="inlineStr">
         <is>
-          <t>Phrasaeng</t>
+          <t>Phunphin</t>
         </is>
       </c>
       <c r="D837" t="n">
@@ -24711,16 +24711,16 @@
     </row>
     <row r="838">
       <c r="A838" t="n">
-        <v>8417</v>
+        <v>8418</v>
       </c>
       <c r="B838" t="inlineStr">
         <is>
-          <t>พุนพิน</t>
+          <t>ชัยบุรี</t>
         </is>
       </c>
       <c r="C838" t="inlineStr">
         <is>
-          <t>Phunphin</t>
+          <t>Chai Buri</t>
         </is>
       </c>
       <c r="D838" t="n">
@@ -24740,16 +24740,16 @@
     </row>
     <row r="839">
       <c r="A839" t="n">
-        <v>8418</v>
+        <v>8419</v>
       </c>
       <c r="B839" t="inlineStr">
         <is>
-          <t>ชัยบุรี</t>
+          <t>วิภาวดี</t>
         </is>
       </c>
       <c r="C839" t="inlineStr">
         <is>
-          <t>Chai Buri</t>
+          <t>Vibhavadi</t>
         </is>
       </c>
       <c r="D839" t="n">
@@ -24769,20 +24769,20 @@
     </row>
     <row r="840">
       <c r="A840" t="n">
-        <v>8419</v>
+        <v>8501</v>
       </c>
       <c r="B840" t="inlineStr">
         <is>
-          <t>วิภาวดี</t>
+          <t>เมืองระนอง</t>
         </is>
       </c>
       <c r="C840" t="inlineStr">
         <is>
-          <t>Vibhavadi</t>
+          <t>Mueang Ranong</t>
         </is>
       </c>
       <c r="D840" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E840" t="inlineStr">
         <is>
@@ -24798,16 +24798,16 @@
     </row>
     <row r="841">
       <c r="A841" t="n">
-        <v>8501</v>
+        <v>8502</v>
       </c>
       <c r="B841" t="inlineStr">
         <is>
-          <t>เมืองระนอง</t>
+          <t>ละอุ่น</t>
         </is>
       </c>
       <c r="C841" t="inlineStr">
         <is>
-          <t>Mueang Ranong</t>
+          <t>La-un</t>
         </is>
       </c>
       <c r="D841" t="n">
@@ -24827,16 +24827,16 @@
     </row>
     <row r="842">
       <c r="A842" t="n">
-        <v>8502</v>
+        <v>8503</v>
       </c>
       <c r="B842" t="inlineStr">
         <is>
-          <t>ละอุ่น</t>
+          <t>กะเปอร์</t>
         </is>
       </c>
       <c r="C842" t="inlineStr">
         <is>
-          <t>La-un</t>
+          <t>Kapoe</t>
         </is>
       </c>
       <c r="D842" t="n">
@@ -24856,16 +24856,16 @@
     </row>
     <row r="843">
       <c r="A843" t="n">
-        <v>8503</v>
+        <v>8504</v>
       </c>
       <c r="B843" t="inlineStr">
         <is>
-          <t>กะเปอร์</t>
+          <t>กระบุรี</t>
         </is>
       </c>
       <c r="C843" t="inlineStr">
         <is>
-          <t>Kapoe</t>
+          <t>Kra Buri</t>
         </is>
       </c>
       <c r="D843" t="n">
@@ -24885,16 +24885,16 @@
     </row>
     <row r="844">
       <c r="A844" t="n">
-        <v>8504</v>
+        <v>8505</v>
       </c>
       <c r="B844" t="inlineStr">
         <is>
-          <t>กระบุรี</t>
+          <t>สุขสำราญ</t>
         </is>
       </c>
       <c r="C844" t="inlineStr">
         <is>
-          <t>Kra Buri</t>
+          <t>Suk Samran</t>
         </is>
       </c>
       <c r="D844" t="n">
@@ -24914,20 +24914,20 @@
     </row>
     <row r="845">
       <c r="A845" t="n">
-        <v>8505</v>
+        <v>8601</v>
       </c>
       <c r="B845" t="inlineStr">
         <is>
-          <t>สุขสำราญ</t>
+          <t>เมืองชุมพร</t>
         </is>
       </c>
       <c r="C845" t="inlineStr">
         <is>
-          <t>Suk Samran</t>
+          <t>Mueang Chumphon</t>
         </is>
       </c>
       <c r="D845" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E845" t="inlineStr">
         <is>
@@ -24943,16 +24943,16 @@
     </row>
     <row r="846">
       <c r="A846" t="n">
-        <v>8601</v>
+        <v>8602</v>
       </c>
       <c r="B846" t="inlineStr">
         <is>
-          <t>เมืองชุมพร</t>
+          <t>ท่าแซะ</t>
         </is>
       </c>
       <c r="C846" t="inlineStr">
         <is>
-          <t>Mueang Chumphon</t>
+          <t>Tha Sae</t>
         </is>
       </c>
       <c r="D846" t="n">
@@ -24972,16 +24972,16 @@
     </row>
     <row r="847">
       <c r="A847" t="n">
-        <v>8602</v>
+        <v>8603</v>
       </c>
       <c r="B847" t="inlineStr">
         <is>
-          <t>ท่าแซะ</t>
+          <t>ปะทิว</t>
         </is>
       </c>
       <c r="C847" t="inlineStr">
         <is>
-          <t>Tha Sae</t>
+          <t>Pathio</t>
         </is>
       </c>
       <c r="D847" t="n">
@@ -25001,16 +25001,16 @@
     </row>
     <row r="848">
       <c r="A848" t="n">
-        <v>8603</v>
+        <v>8604</v>
       </c>
       <c r="B848" t="inlineStr">
         <is>
-          <t>ปะทิว</t>
+          <t>หลังสวน</t>
         </is>
       </c>
       <c r="C848" t="inlineStr">
         <is>
-          <t>Pathio</t>
+          <t>Lang Suan</t>
         </is>
       </c>
       <c r="D848" t="n">
@@ -25030,16 +25030,16 @@
     </row>
     <row r="849">
       <c r="A849" t="n">
-        <v>8604</v>
+        <v>8605</v>
       </c>
       <c r="B849" t="inlineStr">
         <is>
-          <t>หลังสวน</t>
+          <t>ละแม</t>
         </is>
       </c>
       <c r="C849" t="inlineStr">
         <is>
-          <t>Lang Suan</t>
+          <t>Lamae</t>
         </is>
       </c>
       <c r="D849" t="n">
@@ -25059,16 +25059,16 @@
     </row>
     <row r="850">
       <c r="A850" t="n">
-        <v>8605</v>
+        <v>8606</v>
       </c>
       <c r="B850" t="inlineStr">
         <is>
-          <t>ละแม</t>
+          <t>พะโต๊ะ</t>
         </is>
       </c>
       <c r="C850" t="inlineStr">
         <is>
-          <t>Lamae</t>
+          <t>Phato</t>
         </is>
       </c>
       <c r="D850" t="n">
@@ -25088,16 +25088,16 @@
     </row>
     <row r="851">
       <c r="A851" t="n">
-        <v>8606</v>
+        <v>8607</v>
       </c>
       <c r="B851" t="inlineStr">
         <is>
-          <t>พะโต๊ะ</t>
+          <t>สวี</t>
         </is>
       </c>
       <c r="C851" t="inlineStr">
         <is>
-          <t>Phato</t>
+          <t>Sawi</t>
         </is>
       </c>
       <c r="D851" t="n">
@@ -25117,16 +25117,16 @@
     </row>
     <row r="852">
       <c r="A852" t="n">
-        <v>8607</v>
+        <v>8608</v>
       </c>
       <c r="B852" t="inlineStr">
         <is>
-          <t>สวี</t>
+          <t>ทุ่งตะโก</t>
         </is>
       </c>
       <c r="C852" t="inlineStr">
         <is>
-          <t>Sawi</t>
+          <t>Thung Tako</t>
         </is>
       </c>
       <c r="D852" t="n">
@@ -25146,20 +25146,20 @@
     </row>
     <row r="853">
       <c r="A853" t="n">
-        <v>8608</v>
+        <v>9001</v>
       </c>
       <c r="B853" t="inlineStr">
         <is>
-          <t>ทุ่งตะโก</t>
+          <t>เมืองสงขลา</t>
         </is>
       </c>
       <c r="C853" t="inlineStr">
         <is>
-          <t>Thung Tako</t>
+          <t>Mueang Songkhla</t>
         </is>
       </c>
       <c r="D853" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E853" t="inlineStr">
         <is>
@@ -25175,16 +25175,16 @@
     </row>
     <row r="854">
       <c r="A854" t="n">
-        <v>9001</v>
+        <v>9002</v>
       </c>
       <c r="B854" t="inlineStr">
         <is>
-          <t>เมืองสงขลา</t>
+          <t>สทิงพระ</t>
         </is>
       </c>
       <c r="C854" t="inlineStr">
         <is>
-          <t>Mueang Songkhla</t>
+          <t>Sathing Phra</t>
         </is>
       </c>
       <c r="D854" t="n">
@@ -25204,16 +25204,16 @@
     </row>
     <row r="855">
       <c r="A855" t="n">
-        <v>9002</v>
+        <v>9003</v>
       </c>
       <c r="B855" t="inlineStr">
         <is>
-          <t>สทิงพระ</t>
+          <t>จะนะ</t>
         </is>
       </c>
       <c r="C855" t="inlineStr">
         <is>
-          <t>Sathing Phra</t>
+          <t>Chana</t>
         </is>
       </c>
       <c r="D855" t="n">
@@ -25233,16 +25233,16 @@
     </row>
     <row r="856">
       <c r="A856" t="n">
-        <v>9003</v>
+        <v>9004</v>
       </c>
       <c r="B856" t="inlineStr">
         <is>
-          <t>จะนะ</t>
+          <t>นาทวี</t>
         </is>
       </c>
       <c r="C856" t="inlineStr">
         <is>
-          <t>Chana</t>
+          <t>Na Thawi</t>
         </is>
       </c>
       <c r="D856" t="n">
@@ -25262,16 +25262,16 @@
     </row>
     <row r="857">
       <c r="A857" t="n">
-        <v>9004</v>
+        <v>9005</v>
       </c>
       <c r="B857" t="inlineStr">
         <is>
-          <t>นาทวี</t>
+          <t>เทพา</t>
         </is>
       </c>
       <c r="C857" t="inlineStr">
         <is>
-          <t>Na Thawi</t>
+          <t>Thepha</t>
         </is>
       </c>
       <c r="D857" t="n">
@@ -25291,16 +25291,16 @@
     </row>
     <row r="858">
       <c r="A858" t="n">
-        <v>9005</v>
+        <v>9006</v>
       </c>
       <c r="B858" t="inlineStr">
         <is>
-          <t>เทพา</t>
+          <t>สะบ้าย้อย</t>
         </is>
       </c>
       <c r="C858" t="inlineStr">
         <is>
-          <t>Thepha</t>
+          <t>Saba Yoi</t>
         </is>
       </c>
       <c r="D858" t="n">
@@ -25320,16 +25320,16 @@
     </row>
     <row r="859">
       <c r="A859" t="n">
-        <v>9006</v>
+        <v>9007</v>
       </c>
       <c r="B859" t="inlineStr">
         <is>
-          <t>สะบ้าย้อย</t>
+          <t>ระโนด</t>
         </is>
       </c>
       <c r="C859" t="inlineStr">
         <is>
-          <t>Saba Yoi</t>
+          <t>Ranot</t>
         </is>
       </c>
       <c r="D859" t="n">
@@ -25349,16 +25349,16 @@
     </row>
     <row r="860">
       <c r="A860" t="n">
-        <v>9007</v>
+        <v>9008</v>
       </c>
       <c r="B860" t="inlineStr">
         <is>
-          <t>ระโนด</t>
+          <t>กระแสสินธุ์</t>
         </is>
       </c>
       <c r="C860" t="inlineStr">
         <is>
-          <t>Ranot</t>
+          <t>Krasae Sin</t>
         </is>
       </c>
       <c r="D860" t="n">
@@ -25378,16 +25378,16 @@
     </row>
     <row r="861">
       <c r="A861" t="n">
-        <v>9008</v>
+        <v>9009</v>
       </c>
       <c r="B861" t="inlineStr">
         <is>
-          <t>กระแสสินธุ์</t>
+          <t>รัตภูมิ</t>
         </is>
       </c>
       <c r="C861" t="inlineStr">
         <is>
-          <t>Krasae Sin</t>
+          <t>Rattaphum</t>
         </is>
       </c>
       <c r="D861" t="n">
@@ -25407,16 +25407,16 @@
     </row>
     <row r="862">
       <c r="A862" t="n">
-        <v>9009</v>
+        <v>9010</v>
       </c>
       <c r="B862" t="inlineStr">
         <is>
-          <t>รัตภูมิ</t>
+          <t>สะเดา</t>
         </is>
       </c>
       <c r="C862" t="inlineStr">
         <is>
-          <t>Rattaphum</t>
+          <t>Sadao</t>
         </is>
       </c>
       <c r="D862" t="n">
@@ -25436,16 +25436,16 @@
     </row>
     <row r="863">
       <c r="A863" t="n">
-        <v>9010</v>
+        <v>9011</v>
       </c>
       <c r="B863" t="inlineStr">
         <is>
-          <t>สะเดา</t>
+          <t>หาดใหญ่</t>
         </is>
       </c>
       <c r="C863" t="inlineStr">
         <is>
-          <t>Sadao</t>
+          <t>Hat Yai</t>
         </is>
       </c>
       <c r="D863" t="n">
@@ -25465,16 +25465,16 @@
     </row>
     <row r="864">
       <c r="A864" t="n">
-        <v>9011</v>
+        <v>9012</v>
       </c>
       <c r="B864" t="inlineStr">
         <is>
-          <t>หาดใหญ่</t>
+          <t>นาหม่อม</t>
         </is>
       </c>
       <c r="C864" t="inlineStr">
         <is>
-          <t>Hat Yai</t>
+          <t>Na Mom</t>
         </is>
       </c>
       <c r="D864" t="n">
@@ -25494,16 +25494,16 @@
     </row>
     <row r="865">
       <c r="A865" t="n">
-        <v>9012</v>
+        <v>9013</v>
       </c>
       <c r="B865" t="inlineStr">
         <is>
-          <t>นาหม่อม</t>
+          <t>ควนเนียง</t>
         </is>
       </c>
       <c r="C865" t="inlineStr">
         <is>
-          <t>Na Mom</t>
+          <t>Khuan Niang</t>
         </is>
       </c>
       <c r="D865" t="n">
@@ -25523,16 +25523,16 @@
     </row>
     <row r="866">
       <c r="A866" t="n">
-        <v>9013</v>
+        <v>9014</v>
       </c>
       <c r="B866" t="inlineStr">
         <is>
-          <t>ควนเนียง</t>
+          <t>บางกล่ำ</t>
         </is>
       </c>
       <c r="C866" t="inlineStr">
         <is>
-          <t>Khuan Niang</t>
+          <t>Bang Klam</t>
         </is>
       </c>
       <c r="D866" t="n">
@@ -25552,16 +25552,16 @@
     </row>
     <row r="867">
       <c r="A867" t="n">
-        <v>9014</v>
+        <v>9015</v>
       </c>
       <c r="B867" t="inlineStr">
         <is>
-          <t>บางกล่ำ</t>
+          <t>สิงหนคร</t>
         </is>
       </c>
       <c r="C867" t="inlineStr">
         <is>
-          <t>Bang Klam</t>
+          <t>Singhanakhon</t>
         </is>
       </c>
       <c r="D867" t="n">
@@ -25581,16 +25581,16 @@
     </row>
     <row r="868">
       <c r="A868" t="n">
-        <v>9015</v>
+        <v>9016</v>
       </c>
       <c r="B868" t="inlineStr">
         <is>
-          <t>สิงหนคร</t>
+          <t>คลองหอยโข่ง</t>
         </is>
       </c>
       <c r="C868" t="inlineStr">
         <is>
-          <t>Singhanakhon</t>
+          <t>Khlong Hoi Khong</t>
         </is>
       </c>
       <c r="D868" t="n">
@@ -25610,20 +25610,20 @@
     </row>
     <row r="869">
       <c r="A869" t="n">
-        <v>9016</v>
+        <v>9101</v>
       </c>
       <c r="B869" t="inlineStr">
         <is>
-          <t>คลองหอยโข่ง</t>
+          <t>เมืองสตูล</t>
         </is>
       </c>
       <c r="C869" t="inlineStr">
         <is>
-          <t>Khlong Hoi Khong</t>
+          <t>Mueang Satun</t>
         </is>
       </c>
       <c r="D869" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E869" t="inlineStr">
         <is>
@@ -25639,20 +25639,20 @@
     </row>
     <row r="870">
       <c r="A870" t="n">
-        <v>9077</v>
+        <v>9102</v>
       </c>
       <c r="B870" t="inlineStr">
         <is>
-          <t>ท้องถิ่นเทศบาลตำบลสำนักขาม</t>
+          <t>ควนโดน</t>
         </is>
       </c>
       <c r="C870" t="inlineStr">
         <is>
-          <t>Sum Nung Kam</t>
+          <t>Khuan Don</t>
         </is>
       </c>
       <c r="D870" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E870" t="inlineStr">
         <is>
@@ -25668,16 +25668,16 @@
     </row>
     <row r="871">
       <c r="A871" t="n">
-        <v>9101</v>
+        <v>9103</v>
       </c>
       <c r="B871" t="inlineStr">
         <is>
-          <t>เมืองสตูล</t>
+          <t>ควนกาหลง</t>
         </is>
       </c>
       <c r="C871" t="inlineStr">
         <is>
-          <t>Mueang Satun</t>
+          <t>Khuan Kalong</t>
         </is>
       </c>
       <c r="D871" t="n">
@@ -25697,16 +25697,16 @@
     </row>
     <row r="872">
       <c r="A872" t="n">
-        <v>9102</v>
+        <v>9104</v>
       </c>
       <c r="B872" t="inlineStr">
         <is>
-          <t>ควนโดน</t>
+          <t>ท่าแพ</t>
         </is>
       </c>
       <c r="C872" t="inlineStr">
         <is>
-          <t>Khuan Don</t>
+          <t>Tha Phae</t>
         </is>
       </c>
       <c r="D872" t="n">
@@ -25726,16 +25726,16 @@
     </row>
     <row r="873">
       <c r="A873" t="n">
-        <v>9103</v>
+        <v>9105</v>
       </c>
       <c r="B873" t="inlineStr">
         <is>
-          <t>ควนกาหลง</t>
+          <t>ละงู</t>
         </is>
       </c>
       <c r="C873" t="inlineStr">
         <is>
-          <t>Khuan Kalong</t>
+          <t>La-ngu</t>
         </is>
       </c>
       <c r="D873" t="n">
@@ -25755,16 +25755,16 @@
     </row>
     <row r="874">
       <c r="A874" t="n">
-        <v>9104</v>
+        <v>9106</v>
       </c>
       <c r="B874" t="inlineStr">
         <is>
-          <t>ท่าแพ</t>
+          <t>ทุ่งหว้า</t>
         </is>
       </c>
       <c r="C874" t="inlineStr">
         <is>
-          <t>Tha Phae</t>
+          <t>Thung Wa</t>
         </is>
       </c>
       <c r="D874" t="n">
@@ -25784,16 +25784,16 @@
     </row>
     <row r="875">
       <c r="A875" t="n">
-        <v>9105</v>
+        <v>9107</v>
       </c>
       <c r="B875" t="inlineStr">
         <is>
-          <t>ละงู</t>
+          <t>มะนัง</t>
         </is>
       </c>
       <c r="C875" t="inlineStr">
         <is>
-          <t>La-ngu</t>
+          <t>Manang</t>
         </is>
       </c>
       <c r="D875" t="n">
@@ -25813,20 +25813,20 @@
     </row>
     <row r="876">
       <c r="A876" t="n">
-        <v>9106</v>
+        <v>9201</v>
       </c>
       <c r="B876" t="inlineStr">
         <is>
-          <t>ทุ่งหว้า</t>
+          <t>เมืองตรัง</t>
         </is>
       </c>
       <c r="C876" t="inlineStr">
         <is>
-          <t>Thung Wa</t>
+          <t>Mueang Trang</t>
         </is>
       </c>
       <c r="D876" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E876" t="inlineStr">
         <is>
@@ -25842,20 +25842,20 @@
     </row>
     <row r="877">
       <c r="A877" t="n">
-        <v>9107</v>
+        <v>9202</v>
       </c>
       <c r="B877" t="inlineStr">
         <is>
-          <t>มะนัง</t>
+          <t>กันตัง</t>
         </is>
       </c>
       <c r="C877" t="inlineStr">
         <is>
-          <t>Manang</t>
+          <t>Kantang</t>
         </is>
       </c>
       <c r="D877" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E877" t="inlineStr">
         <is>
@@ -25871,16 +25871,16 @@
     </row>
     <row r="878">
       <c r="A878" t="n">
-        <v>9201</v>
+        <v>9203</v>
       </c>
       <c r="B878" t="inlineStr">
         <is>
-          <t>เมืองตรัง</t>
+          <t>ย่านตาขาว</t>
         </is>
       </c>
       <c r="C878" t="inlineStr">
         <is>
-          <t>Mueang Trang</t>
+          <t>Yan Ta Khao</t>
         </is>
       </c>
       <c r="D878" t="n">
@@ -25900,16 +25900,16 @@
     </row>
     <row r="879">
       <c r="A879" t="n">
-        <v>9202</v>
+        <v>9204</v>
       </c>
       <c r="B879" t="inlineStr">
         <is>
-          <t>กันตัง</t>
+          <t>ปะเหลียน</t>
         </is>
       </c>
       <c r="C879" t="inlineStr">
         <is>
-          <t>Kantang</t>
+          <t>Palian</t>
         </is>
       </c>
       <c r="D879" t="n">
@@ -25929,16 +25929,16 @@
     </row>
     <row r="880">
       <c r="A880" t="n">
-        <v>9203</v>
+        <v>9205</v>
       </c>
       <c r="B880" t="inlineStr">
         <is>
-          <t>ย่านตาขาว</t>
+          <t>สิเกา</t>
         </is>
       </c>
       <c r="C880" t="inlineStr">
         <is>
-          <t>Yan Ta Khao</t>
+          <t>Sikao</t>
         </is>
       </c>
       <c r="D880" t="n">
@@ -25958,16 +25958,16 @@
     </row>
     <row r="881">
       <c r="A881" t="n">
-        <v>9204</v>
+        <v>9206</v>
       </c>
       <c r="B881" t="inlineStr">
         <is>
-          <t>ปะเหลียน</t>
+          <t>ห้วยยอด</t>
         </is>
       </c>
       <c r="C881" t="inlineStr">
         <is>
-          <t>Palian</t>
+          <t>Huai Yot</t>
         </is>
       </c>
       <c r="D881" t="n">
@@ -25987,16 +25987,16 @@
     </row>
     <row r="882">
       <c r="A882" t="n">
-        <v>9205</v>
+        <v>9207</v>
       </c>
       <c r="B882" t="inlineStr">
         <is>
-          <t>สิเกา</t>
+          <t>วังวิเศษ</t>
         </is>
       </c>
       <c r="C882" t="inlineStr">
         <is>
-          <t>Sikao</t>
+          <t>Wang Wiset</t>
         </is>
       </c>
       <c r="D882" t="n">
@@ -26016,16 +26016,16 @@
     </row>
     <row r="883">
       <c r="A883" t="n">
-        <v>9206</v>
+        <v>9208</v>
       </c>
       <c r="B883" t="inlineStr">
         <is>
-          <t>ห้วยยอด</t>
+          <t>นาโยง</t>
         </is>
       </c>
       <c r="C883" t="inlineStr">
         <is>
-          <t>Huai Yot</t>
+          <t>Na Yong</t>
         </is>
       </c>
       <c r="D883" t="n">
@@ -26045,16 +26045,16 @@
     </row>
     <row r="884">
       <c r="A884" t="n">
-        <v>9207</v>
+        <v>9209</v>
       </c>
       <c r="B884" t="inlineStr">
         <is>
-          <t>วังวิเศษ</t>
+          <t>รัษฎา</t>
         </is>
       </c>
       <c r="C884" t="inlineStr">
         <is>
-          <t>Wang Wiset</t>
+          <t>Ratsada</t>
         </is>
       </c>
       <c r="D884" t="n">
@@ -26074,16 +26074,16 @@
     </row>
     <row r="885">
       <c r="A885" t="n">
-        <v>9208</v>
+        <v>9210</v>
       </c>
       <c r="B885" t="inlineStr">
         <is>
-          <t>นาโยง</t>
+          <t>หาดสำราญ</t>
         </is>
       </c>
       <c r="C885" t="inlineStr">
         <is>
-          <t>Na Yong</t>
+          <t>Hat Samran</t>
         </is>
       </c>
       <c r="D885" t="n">
@@ -26103,20 +26103,20 @@
     </row>
     <row r="886">
       <c r="A886" t="n">
-        <v>9209</v>
+        <v>9301</v>
       </c>
       <c r="B886" t="inlineStr">
         <is>
-          <t>รัษฎา</t>
+          <t>เมืองพัทลุง</t>
         </is>
       </c>
       <c r="C886" t="inlineStr">
         <is>
-          <t>Ratsada</t>
+          <t>Mueang Phatthalung</t>
         </is>
       </c>
       <c r="D886" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E886" t="inlineStr">
         <is>
@@ -26132,20 +26132,20 @@
     </row>
     <row r="887">
       <c r="A887" t="n">
-        <v>9210</v>
+        <v>9302</v>
       </c>
       <c r="B887" t="inlineStr">
         <is>
-          <t>หาดสำราญ</t>
+          <t>กงหรา</t>
         </is>
       </c>
       <c r="C887" t="inlineStr">
         <is>
-          <t>Hat Samran</t>
+          <t>Kong Ra</t>
         </is>
       </c>
       <c r="D887" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E887" t="inlineStr">
         <is>
@@ -26161,16 +26161,16 @@
     </row>
     <row r="888">
       <c r="A888" t="n">
-        <v>9301</v>
+        <v>9303</v>
       </c>
       <c r="B888" t="inlineStr">
         <is>
-          <t>เมืองพัทลุง</t>
+          <t>เขาชัยสน</t>
         </is>
       </c>
       <c r="C888" t="inlineStr">
         <is>
-          <t>Mueang Phatthalung</t>
+          <t>Khao Chaison</t>
         </is>
       </c>
       <c r="D888" t="n">
@@ -26190,16 +26190,16 @@
     </row>
     <row r="889">
       <c r="A889" t="n">
-        <v>9302</v>
+        <v>9304</v>
       </c>
       <c r="B889" t="inlineStr">
         <is>
-          <t>กงหรา</t>
+          <t>ตะโหมด</t>
         </is>
       </c>
       <c r="C889" t="inlineStr">
         <is>
-          <t>Kong Ra</t>
+          <t>Tamot</t>
         </is>
       </c>
       <c r="D889" t="n">
@@ -26219,16 +26219,16 @@
     </row>
     <row r="890">
       <c r="A890" t="n">
-        <v>9303</v>
+        <v>9305</v>
       </c>
       <c r="B890" t="inlineStr">
         <is>
-          <t>เขาชัยสน</t>
+          <t>ควนขนุน</t>
         </is>
       </c>
       <c r="C890" t="inlineStr">
         <is>
-          <t>Khao Chaison</t>
+          <t>Khuan Khanun</t>
         </is>
       </c>
       <c r="D890" t="n">
@@ -26248,16 +26248,16 @@
     </row>
     <row r="891">
       <c r="A891" t="n">
-        <v>9304</v>
+        <v>9306</v>
       </c>
       <c r="B891" t="inlineStr">
         <is>
-          <t>ตะโหมด</t>
+          <t>ปากพะยูน</t>
         </is>
       </c>
       <c r="C891" t="inlineStr">
         <is>
-          <t>Tamot</t>
+          <t>Pak Phayun</t>
         </is>
       </c>
       <c r="D891" t="n">
@@ -26277,16 +26277,16 @@
     </row>
     <row r="892">
       <c r="A892" t="n">
-        <v>9305</v>
+        <v>9307</v>
       </c>
       <c r="B892" t="inlineStr">
         <is>
-          <t>ควนขนุน</t>
+          <t>ศรีบรรพต</t>
         </is>
       </c>
       <c r="C892" t="inlineStr">
         <is>
-          <t>Khuan Khanun</t>
+          <t>Si Banphot</t>
         </is>
       </c>
       <c r="D892" t="n">
@@ -26306,16 +26306,16 @@
     </row>
     <row r="893">
       <c r="A893" t="n">
-        <v>9306</v>
+        <v>9308</v>
       </c>
       <c r="B893" t="inlineStr">
         <is>
-          <t>ปากพะยูน</t>
+          <t>ป่าบอน</t>
         </is>
       </c>
       <c r="C893" t="inlineStr">
         <is>
-          <t>Pak Phayun</t>
+          <t>Pa Bon</t>
         </is>
       </c>
       <c r="D893" t="n">
@@ -26335,16 +26335,16 @@
     </row>
     <row r="894">
       <c r="A894" t="n">
-        <v>9307</v>
+        <v>9309</v>
       </c>
       <c r="B894" t="inlineStr">
         <is>
-          <t>ศรีบรรพต</t>
+          <t>บางแก้ว</t>
         </is>
       </c>
       <c r="C894" t="inlineStr">
         <is>
-          <t>Si Banphot</t>
+          <t>Bang Kaeo</t>
         </is>
       </c>
       <c r="D894" t="n">
@@ -26364,16 +26364,16 @@
     </row>
     <row r="895">
       <c r="A895" t="n">
-        <v>9308</v>
+        <v>9310</v>
       </c>
       <c r="B895" t="inlineStr">
         <is>
-          <t>ป่าบอน</t>
+          <t>ป่าพะยอม</t>
         </is>
       </c>
       <c r="C895" t="inlineStr">
         <is>
-          <t>Pa Bon</t>
+          <t>Pa Phayom</t>
         </is>
       </c>
       <c r="D895" t="n">
@@ -26393,16 +26393,16 @@
     </row>
     <row r="896">
       <c r="A896" t="n">
-        <v>9309</v>
+        <v>9311</v>
       </c>
       <c r="B896" t="inlineStr">
         <is>
-          <t>บางแก้ว</t>
+          <t>ศรีนครินทร์</t>
         </is>
       </c>
       <c r="C896" t="inlineStr">
         <is>
-          <t>Bang Kaeo</t>
+          <t>Srinagarindra</t>
         </is>
       </c>
       <c r="D896" t="n">
@@ -26422,20 +26422,20 @@
     </row>
     <row r="897">
       <c r="A897" t="n">
-        <v>9310</v>
+        <v>9401</v>
       </c>
       <c r="B897" t="inlineStr">
         <is>
-          <t>ป่าพะยอม</t>
+          <t>เมืองปัตตานี</t>
         </is>
       </c>
       <c r="C897" t="inlineStr">
         <is>
-          <t>Pa Phayom</t>
+          <t>Mueang Pattani</t>
         </is>
       </c>
       <c r="D897" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E897" t="inlineStr">
         <is>
@@ -26451,20 +26451,20 @@
     </row>
     <row r="898">
       <c r="A898" t="n">
-        <v>9311</v>
+        <v>9402</v>
       </c>
       <c r="B898" t="inlineStr">
         <is>
-          <t>ศรีนครินทร์</t>
+          <t>โคกโพธิ์</t>
         </is>
       </c>
       <c r="C898" t="inlineStr">
         <is>
-          <t>Srinagarindra</t>
+          <t>Khok Pho</t>
         </is>
       </c>
       <c r="D898" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E898" t="inlineStr">
         <is>
@@ -26480,16 +26480,16 @@
     </row>
     <row r="899">
       <c r="A899" t="n">
-        <v>9401</v>
+        <v>9403</v>
       </c>
       <c r="B899" t="inlineStr">
         <is>
-          <t>เมืองปัตตานี</t>
+          <t>หนองจิก</t>
         </is>
       </c>
       <c r="C899" t="inlineStr">
         <is>
-          <t>Mueang Pattani</t>
+          <t>Nong Chik</t>
         </is>
       </c>
       <c r="D899" t="n">
@@ -26509,16 +26509,16 @@
     </row>
     <row r="900">
       <c r="A900" t="n">
-        <v>9402</v>
+        <v>9404</v>
       </c>
       <c r="B900" t="inlineStr">
         <is>
-          <t>โคกโพธิ์</t>
+          <t>ปะนาเระ</t>
         </is>
       </c>
       <c r="C900" t="inlineStr">
         <is>
-          <t>Khok Pho</t>
+          <t>Panare</t>
         </is>
       </c>
       <c r="D900" t="n">
@@ -26538,16 +26538,16 @@
     </row>
     <row r="901">
       <c r="A901" t="n">
-        <v>9403</v>
+        <v>9405</v>
       </c>
       <c r="B901" t="inlineStr">
         <is>
-          <t>หนองจิก</t>
+          <t>มายอ</t>
         </is>
       </c>
       <c r="C901" t="inlineStr">
         <is>
-          <t>Nong Chik</t>
+          <t>Mayo</t>
         </is>
       </c>
       <c r="D901" t="n">
@@ -26567,16 +26567,16 @@
     </row>
     <row r="902">
       <c r="A902" t="n">
-        <v>9404</v>
+        <v>9406</v>
       </c>
       <c r="B902" t="inlineStr">
         <is>
-          <t>ปะนาเระ</t>
+          <t>ทุ่งยางแดง</t>
         </is>
       </c>
       <c r="C902" t="inlineStr">
         <is>
-          <t>Panare</t>
+          <t>Thung Yang Daeng</t>
         </is>
       </c>
       <c r="D902" t="n">
@@ -26596,16 +26596,16 @@
     </row>
     <row r="903">
       <c r="A903" t="n">
-        <v>9405</v>
+        <v>9407</v>
       </c>
       <c r="B903" t="inlineStr">
         <is>
-          <t>มายอ</t>
+          <t>สายบุรี</t>
         </is>
       </c>
       <c r="C903" t="inlineStr">
         <is>
-          <t>Mayo</t>
+          <t>Sai Buri</t>
         </is>
       </c>
       <c r="D903" t="n">
@@ -26625,16 +26625,16 @@
     </row>
     <row r="904">
       <c r="A904" t="n">
-        <v>9406</v>
+        <v>9408</v>
       </c>
       <c r="B904" t="inlineStr">
         <is>
-          <t>ทุ่งยางแดง</t>
+          <t>ไม้แก่น</t>
         </is>
       </c>
       <c r="C904" t="inlineStr">
         <is>
-          <t>Thung Yang Daeng</t>
+          <t>Mai Kaen</t>
         </is>
       </c>
       <c r="D904" t="n">
@@ -26654,16 +26654,16 @@
     </row>
     <row r="905">
       <c r="A905" t="n">
-        <v>9407</v>
+        <v>9409</v>
       </c>
       <c r="B905" t="inlineStr">
         <is>
-          <t>สายบุรี</t>
+          <t>ยะหริ่ง</t>
         </is>
       </c>
       <c r="C905" t="inlineStr">
         <is>
-          <t>Sai Buri</t>
+          <t>Yaring</t>
         </is>
       </c>
       <c r="D905" t="n">
@@ -26683,16 +26683,16 @@
     </row>
     <row r="906">
       <c r="A906" t="n">
-        <v>9408</v>
+        <v>9410</v>
       </c>
       <c r="B906" t="inlineStr">
         <is>
-          <t>ไม้แก่น</t>
+          <t>ยะรัง</t>
         </is>
       </c>
       <c r="C906" t="inlineStr">
         <is>
-          <t>Mai Kaen</t>
+          <t>Yarang</t>
         </is>
       </c>
       <c r="D906" t="n">
@@ -26712,16 +26712,16 @@
     </row>
     <row r="907">
       <c r="A907" t="n">
-        <v>9409</v>
+        <v>9411</v>
       </c>
       <c r="B907" t="inlineStr">
         <is>
-          <t>ยะหริ่ง</t>
+          <t>กะพ้อ</t>
         </is>
       </c>
       <c r="C907" t="inlineStr">
         <is>
-          <t>Yaring</t>
+          <t>Kapho</t>
         </is>
       </c>
       <c r="D907" t="n">
@@ -26741,16 +26741,16 @@
     </row>
     <row r="908">
       <c r="A908" t="n">
-        <v>9410</v>
+        <v>9412</v>
       </c>
       <c r="B908" t="inlineStr">
         <is>
-          <t>ยะรัง</t>
+          <t>แม่ลาน</t>
         </is>
       </c>
       <c r="C908" t="inlineStr">
         <is>
-          <t>Yarang</t>
+          <t>Mae Lan</t>
         </is>
       </c>
       <c r="D908" t="n">
@@ -26770,20 +26770,20 @@
     </row>
     <row r="909">
       <c r="A909" t="n">
-        <v>9411</v>
+        <v>9501</v>
       </c>
       <c r="B909" t="inlineStr">
         <is>
-          <t>กะพ้อ</t>
+          <t>เมืองยะลา</t>
         </is>
       </c>
       <c r="C909" t="inlineStr">
         <is>
-          <t>Kapho</t>
+          <t>Mueang Yala</t>
         </is>
       </c>
       <c r="D909" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E909" t="inlineStr">
         <is>
@@ -26799,20 +26799,20 @@
     </row>
     <row r="910">
       <c r="A910" t="n">
-        <v>9412</v>
+        <v>9502</v>
       </c>
       <c r="B910" t="inlineStr">
         <is>
-          <t>แม่ลาน</t>
+          <t>เบตง</t>
         </is>
       </c>
       <c r="C910" t="inlineStr">
         <is>
-          <t>Mae Lan</t>
+          <t>Betong</t>
         </is>
       </c>
       <c r="D910" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E910" t="inlineStr">
         <is>
@@ -26828,16 +26828,16 @@
     </row>
     <row r="911">
       <c r="A911" t="n">
-        <v>9501</v>
+        <v>9503</v>
       </c>
       <c r="B911" t="inlineStr">
         <is>
-          <t>เมืองยะลา</t>
+          <t>บันนังสตา</t>
         </is>
       </c>
       <c r="C911" t="inlineStr">
         <is>
-          <t>Mueang Yala</t>
+          <t>Bannang Sata</t>
         </is>
       </c>
       <c r="D911" t="n">
@@ -26857,16 +26857,16 @@
     </row>
     <row r="912">
       <c r="A912" t="n">
-        <v>9502</v>
+        <v>9504</v>
       </c>
       <c r="B912" t="inlineStr">
         <is>
-          <t>เบตง</t>
+          <t>ธารโต</t>
         </is>
       </c>
       <c r="C912" t="inlineStr">
         <is>
-          <t>Betong</t>
+          <t>Than To</t>
         </is>
       </c>
       <c r="D912" t="n">
@@ -26886,16 +26886,16 @@
     </row>
     <row r="913">
       <c r="A913" t="n">
-        <v>9503</v>
+        <v>9505</v>
       </c>
       <c r="B913" t="inlineStr">
         <is>
-          <t>บันนังสตา</t>
+          <t>ยะหา</t>
         </is>
       </c>
       <c r="C913" t="inlineStr">
         <is>
-          <t>Bannang Sata</t>
+          <t>Yaha</t>
         </is>
       </c>
       <c r="D913" t="n">
@@ -26915,16 +26915,16 @@
     </row>
     <row r="914">
       <c r="A914" t="n">
-        <v>9504</v>
+        <v>9506</v>
       </c>
       <c r="B914" t="inlineStr">
         <is>
-          <t>ธารโต</t>
+          <t>รามัน</t>
         </is>
       </c>
       <c r="C914" t="inlineStr">
         <is>
-          <t>Than To</t>
+          <t>Raman</t>
         </is>
       </c>
       <c r="D914" t="n">
@@ -26944,16 +26944,16 @@
     </row>
     <row r="915">
       <c r="A915" t="n">
-        <v>9505</v>
+        <v>9507</v>
       </c>
       <c r="B915" t="inlineStr">
         <is>
-          <t>ยะหา</t>
+          <t>กาบัง</t>
         </is>
       </c>
       <c r="C915" t="inlineStr">
         <is>
-          <t>Yaha</t>
+          <t>Kabang</t>
         </is>
       </c>
       <c r="D915" t="n">
@@ -26973,16 +26973,16 @@
     </row>
     <row r="916">
       <c r="A916" t="n">
-        <v>9506</v>
+        <v>9508</v>
       </c>
       <c r="B916" t="inlineStr">
         <is>
-          <t>รามัน</t>
+          <t>กรงปินัง</t>
         </is>
       </c>
       <c r="C916" t="inlineStr">
         <is>
-          <t>Raman</t>
+          <t>Krong Pinang</t>
         </is>
       </c>
       <c r="D916" t="n">
@@ -27002,20 +27002,20 @@
     </row>
     <row r="917">
       <c r="A917" t="n">
-        <v>9507</v>
+        <v>9601</v>
       </c>
       <c r="B917" t="inlineStr">
         <is>
-          <t>กาบัง</t>
+          <t>เมืองนราธิวาส</t>
         </is>
       </c>
       <c r="C917" t="inlineStr">
         <is>
-          <t>Kabang</t>
+          <t>Mueang Narathiwat</t>
         </is>
       </c>
       <c r="D917" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E917" t="inlineStr">
         <is>
@@ -27031,20 +27031,20 @@
     </row>
     <row r="918">
       <c r="A918" t="n">
-        <v>9508</v>
+        <v>9602</v>
       </c>
       <c r="B918" t="inlineStr">
         <is>
-          <t>กรงปินัง</t>
+          <t>ตากใบ</t>
         </is>
       </c>
       <c r="C918" t="inlineStr">
         <is>
-          <t>Krong Pinang</t>
+          <t>Tak Bai</t>
         </is>
       </c>
       <c r="D918" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E918" t="inlineStr">
         <is>
@@ -27060,16 +27060,16 @@
     </row>
     <row r="919">
       <c r="A919" t="n">
-        <v>9601</v>
+        <v>9603</v>
       </c>
       <c r="B919" t="inlineStr">
         <is>
-          <t>เมืองนราธิวาส</t>
+          <t>บาเจาะ</t>
         </is>
       </c>
       <c r="C919" t="inlineStr">
         <is>
-          <t>Mueang Narathiwat</t>
+          <t>Bacho</t>
         </is>
       </c>
       <c r="D919" t="n">
@@ -27089,16 +27089,16 @@
     </row>
     <row r="920">
       <c r="A920" t="n">
-        <v>9602</v>
+        <v>9604</v>
       </c>
       <c r="B920" t="inlineStr">
         <is>
-          <t>ตากใบ</t>
+          <t>ยี่งอ</t>
         </is>
       </c>
       <c r="C920" t="inlineStr">
         <is>
-          <t>Tak Bai</t>
+          <t>Yi-ngo</t>
         </is>
       </c>
       <c r="D920" t="n">
@@ -27118,16 +27118,16 @@
     </row>
     <row r="921">
       <c r="A921" t="n">
-        <v>9603</v>
+        <v>9605</v>
       </c>
       <c r="B921" t="inlineStr">
         <is>
-          <t>บาเจาะ</t>
+          <t>ระแงะ</t>
         </is>
       </c>
       <c r="C921" t="inlineStr">
         <is>
-          <t>Bacho</t>
+          <t>Ra-ngae</t>
         </is>
       </c>
       <c r="D921" t="n">
@@ -27147,16 +27147,16 @@
     </row>
     <row r="922">
       <c r="A922" t="n">
-        <v>9604</v>
+        <v>9606</v>
       </c>
       <c r="B922" t="inlineStr">
         <is>
-          <t>ยี่งอ</t>
+          <t>รือเสาะ</t>
         </is>
       </c>
       <c r="C922" t="inlineStr">
         <is>
-          <t>Yi-ngo</t>
+          <t>Rueso</t>
         </is>
       </c>
       <c r="D922" t="n">
@@ -27176,16 +27176,16 @@
     </row>
     <row r="923">
       <c r="A923" t="n">
-        <v>9605</v>
+        <v>9607</v>
       </c>
       <c r="B923" t="inlineStr">
         <is>
-          <t>ระแงะ</t>
+          <t>ศรีสาคร</t>
         </is>
       </c>
       <c r="C923" t="inlineStr">
         <is>
-          <t>Ra-ngae</t>
+          <t>Si Sakhon</t>
         </is>
       </c>
       <c r="D923" t="n">
@@ -27205,16 +27205,16 @@
     </row>
     <row r="924">
       <c r="A924" t="n">
-        <v>9606</v>
+        <v>9608</v>
       </c>
       <c r="B924" t="inlineStr">
         <is>
-          <t>รือเสาะ</t>
+          <t>แว้ง</t>
         </is>
       </c>
       <c r="C924" t="inlineStr">
         <is>
-          <t>Rueso</t>
+          <t>Waeng</t>
         </is>
       </c>
       <c r="D924" t="n">
@@ -27234,16 +27234,16 @@
     </row>
     <row r="925">
       <c r="A925" t="n">
-        <v>9607</v>
+        <v>9609</v>
       </c>
       <c r="B925" t="inlineStr">
         <is>
-          <t>ศรีสาคร</t>
+          <t>สุคิริน</t>
         </is>
       </c>
       <c r="C925" t="inlineStr">
         <is>
-          <t>Si Sakhon</t>
+          <t>Sukhirin</t>
         </is>
       </c>
       <c r="D925" t="n">
@@ -27263,16 +27263,16 @@
     </row>
     <row r="926">
       <c r="A926" t="n">
-        <v>9608</v>
+        <v>9610</v>
       </c>
       <c r="B926" t="inlineStr">
         <is>
-          <t>แว้ง</t>
+          <t>สุไหงโก-ลก</t>
         </is>
       </c>
       <c r="C926" t="inlineStr">
         <is>
-          <t>Waeng</t>
+          <t>Su-ngai Kolok</t>
         </is>
       </c>
       <c r="D926" t="n">
@@ -27292,16 +27292,16 @@
     </row>
     <row r="927">
       <c r="A927" t="n">
-        <v>9609</v>
+        <v>9611</v>
       </c>
       <c r="B927" t="inlineStr">
         <is>
-          <t>สุคิริน</t>
+          <t>สุไหงปาดี</t>
         </is>
       </c>
       <c r="C927" t="inlineStr">
         <is>
-          <t>Sukhirin</t>
+          <t>Su-ngai Padi</t>
         </is>
       </c>
       <c r="D927" t="n">
@@ -27321,16 +27321,16 @@
     </row>
     <row r="928">
       <c r="A928" t="n">
-        <v>9610</v>
+        <v>9612</v>
       </c>
       <c r="B928" t="inlineStr">
         <is>
-          <t>สุไหงโก-ลก</t>
+          <t>จะแนะ</t>
         </is>
       </c>
       <c r="C928" t="inlineStr">
         <is>
-          <t>Su-ngai Kolok</t>
+          <t>Chanae</t>
         </is>
       </c>
       <c r="D928" t="n">
@@ -27350,16 +27350,16 @@
     </row>
     <row r="929">
       <c r="A929" t="n">
-        <v>9611</v>
+        <v>9613</v>
       </c>
       <c r="B929" t="inlineStr">
         <is>
-          <t>สุไหงปาดี</t>
+          <t>เจาะไอร้อง</t>
         </is>
       </c>
       <c r="C929" t="inlineStr">
         <is>
-          <t>Su-ngai Padi</t>
+          <t>Cho-airong</t>
         </is>
       </c>
       <c r="D929" t="n">
@@ -27376,64 +27376,6 @@
         </is>
       </c>
       <c r="G929" t="inlineStr"/>
-    </row>
-    <row r="930">
-      <c r="A930" t="n">
-        <v>9612</v>
-      </c>
-      <c r="B930" t="inlineStr">
-        <is>
-          <t>จะแนะ</t>
-        </is>
-      </c>
-      <c r="C930" t="inlineStr">
-        <is>
-          <t>Chanae</t>
-        </is>
-      </c>
-      <c r="D930" t="n">
-        <v>76</v>
-      </c>
-      <c r="E930" t="inlineStr">
-        <is>
-          <t>2019-08-09T03:33:09.000+07:00</t>
-        </is>
-      </c>
-      <c r="F930" t="inlineStr">
-        <is>
-          <t>2025-09-20T06:31:26.000+07:00</t>
-        </is>
-      </c>
-      <c r="G930" t="inlineStr"/>
-    </row>
-    <row r="931">
-      <c r="A931" t="n">
-        <v>9613</v>
-      </c>
-      <c r="B931" t="inlineStr">
-        <is>
-          <t>เจาะไอร้อง</t>
-        </is>
-      </c>
-      <c r="C931" t="inlineStr">
-        <is>
-          <t>Cho-airong</t>
-        </is>
-      </c>
-      <c r="D931" t="n">
-        <v>76</v>
-      </c>
-      <c r="E931" t="inlineStr">
-        <is>
-          <t>2019-08-09T03:33:09.000+07:00</t>
-        </is>
-      </c>
-      <c r="F931" t="inlineStr">
-        <is>
-          <t>2025-09-20T06:31:26.000+07:00</t>
-        </is>
-      </c>
-      <c r="G931" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>